<commit_message>
test: add E2E test cases for spoiled items freshness checks and logo branding consistency
</commit_message>
<xml_diff>
--- a/testing/reports/web_e2e_report.xlsx
+++ b/testing/reports/web_e2e_report.xlsx
@@ -430,7 +430,7 @@
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>2026-08-24T17:51:03.372Z</v>
+        <v>2026-08-26T05:27:38.356Z</v>
       </c>
     </row>
     <row r="3">
@@ -447,7 +447,7 @@
         <v/>
       </c>
       <c r="E3" t="str">
-        <v>2026-08-24T17:51:04.313Z</v>
+        <v>2026-08-26T05:27:38.821Z</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -462,10 +462,10 @@
       </c>
       <c r="D4" t="str" xml:space="preserve">
         <v xml:space="preserve">Waiting for title to contain "FreshRadar"
-Wait timed out after 60063ms</v>
+Wait timed out after 60045ms</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-08-24T17:52:04.379Z</v>
+        <v>2026-08-26T05:28:38.866Z</v>
       </c>
     </row>
     <row r="5">
@@ -482,7 +482,7 @@
         <v/>
       </c>
       <c r="E5" t="str">
-        <v>2026-08-24T17:52:04.506Z</v>
+        <v>2026-08-26T05:28:39.004Z</v>
       </c>
     </row>
     <row r="6">
@@ -499,7 +499,7 @@
         <v/>
       </c>
       <c r="E6" t="str">
-        <v>2026-08-24T17:52:04.506Z</v>
+        <v>2026-08-26T05:28:39.004Z</v>
       </c>
     </row>
     <row r="7">
@@ -516,7 +516,7 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>2026-08-24T17:52:04.506Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="8">
@@ -533,7 +533,7 @@
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>2026-08-24T17:52:04.506Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="9">
@@ -550,7 +550,7 @@
         <v/>
       </c>
       <c r="E9" t="str">
-        <v>2026-08-24T17:52:04.506Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="10">
@@ -567,7 +567,7 @@
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>2026-08-24T17:52:04.506Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="11">
@@ -584,7 +584,7 @@
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>2026-08-24T17:52:04.506Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="12">
@@ -601,7 +601,7 @@
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>2026-08-24T17:52:04.506Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="13">
@@ -618,7 +618,7 @@
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>2026-08-24T17:52:04.506Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="14">
@@ -635,7 +635,7 @@
         <v/>
       </c>
       <c r="E14" t="str">
-        <v>2026-08-24T17:52:04.506Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="15">
@@ -652,7 +652,7 @@
         <v/>
       </c>
       <c r="E15" t="str">
-        <v>2026-08-24T17:52:04.506Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="16">
@@ -669,7 +669,7 @@
         <v/>
       </c>
       <c r="E16" t="str">
-        <v>2026-08-24T17:52:04.506Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="17">
@@ -686,7 +686,7 @@
         <v/>
       </c>
       <c r="E17" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="18">
@@ -703,7 +703,7 @@
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="19">
@@ -720,7 +720,7 @@
         <v/>
       </c>
       <c r="E19" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="20">
@@ -737,7 +737,7 @@
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="21">
@@ -754,7 +754,7 @@
         <v/>
       </c>
       <c r="E21" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="22">
@@ -771,7 +771,7 @@
         <v/>
       </c>
       <c r="E22" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="23">
@@ -788,7 +788,7 @@
         <v/>
       </c>
       <c r="E23" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="24">
@@ -805,7 +805,7 @@
         <v/>
       </c>
       <c r="E24" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="25">
@@ -822,7 +822,7 @@
         <v/>
       </c>
       <c r="E25" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="26">
@@ -839,7 +839,7 @@
         <v/>
       </c>
       <c r="E26" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="27">
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="E27" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="28">
@@ -873,7 +873,7 @@
         <v/>
       </c>
       <c r="E28" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="29">
@@ -890,7 +890,7 @@
         <v/>
       </c>
       <c r="E29" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="30">
@@ -907,7 +907,7 @@
         <v/>
       </c>
       <c r="E30" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.005Z</v>
       </c>
     </row>
     <row r="31">
@@ -924,7 +924,7 @@
         <v/>
       </c>
       <c r="E31" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="32">
@@ -941,7 +941,7 @@
         <v/>
       </c>
       <c r="E32" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="33">
@@ -958,7 +958,7 @@
         <v/>
       </c>
       <c r="E33" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="34">
@@ -975,7 +975,7 @@
         <v/>
       </c>
       <c r="E34" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="35">
@@ -992,7 +992,7 @@
         <v/>
       </c>
       <c r="E35" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="36">
@@ -1009,7 +1009,7 @@
         <v/>
       </c>
       <c r="E36" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="37">
@@ -1026,7 +1026,7 @@
         <v/>
       </c>
       <c r="E37" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="38">
@@ -1043,7 +1043,7 @@
         <v/>
       </c>
       <c r="E38" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="39">
@@ -1060,7 +1060,7 @@
         <v/>
       </c>
       <c r="E39" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="40">
@@ -1077,7 +1077,7 @@
         <v/>
       </c>
       <c r="E40" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="41">
@@ -1094,7 +1094,7 @@
         <v/>
       </c>
       <c r="E41" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="42">
@@ -1111,7 +1111,7 @@
         <v/>
       </c>
       <c r="E42" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="43">
@@ -1128,7 +1128,7 @@
         <v/>
       </c>
       <c r="E43" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="44">
@@ -1145,7 +1145,7 @@
         <v/>
       </c>
       <c r="E44" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="45">
@@ -1162,7 +1162,7 @@
         <v/>
       </c>
       <c r="E45" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="46">
@@ -1179,7 +1179,7 @@
         <v/>
       </c>
       <c r="E46" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="47">
@@ -1196,7 +1196,7 @@
         <v/>
       </c>
       <c r="E47" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="48">
@@ -1213,7 +1213,7 @@
         <v/>
       </c>
       <c r="E48" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="49">
@@ -1230,7 +1230,7 @@
         <v/>
       </c>
       <c r="E49" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="50">
@@ -1247,7 +1247,7 @@
         <v/>
       </c>
       <c r="E50" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="51">
@@ -1264,7 +1264,7 @@
         <v/>
       </c>
       <c r="E51" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="52">
@@ -1281,7 +1281,7 @@
         <v/>
       </c>
       <c r="E52" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="53">
@@ -1298,7 +1298,7 @@
         <v/>
       </c>
       <c r="E53" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="54">
@@ -1315,7 +1315,7 @@
         <v/>
       </c>
       <c r="E54" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="55">
@@ -1323,7 +1323,7 @@
         <v>TS-WEB-054</v>
       </c>
       <c r="B55" t="str">
-        <v>Verify navbar navigation to Dashboard [Browser: Firefox]</v>
+        <v>Verify items with &lt;= 50% freshness have Used/Not Used actions hidden on web [Browser: Chrome]</v>
       </c>
       <c r="C55" t="str">
         <v>Passed</v>
@@ -1332,7 +1332,7 @@
         <v/>
       </c>
       <c r="E55" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="56">
@@ -1340,7 +1340,7 @@
         <v>TS-WEB-055</v>
       </c>
       <c r="B56" t="str">
-        <v>Verify navbar navigation to Inventory [Browser: Firefox]</v>
+        <v>Verify items with &lt;= 50% freshness do not generate web recipe recommendations [Browser: Chrome]</v>
       </c>
       <c r="C56" t="str">
         <v>Passed</v>
@@ -1349,7 +1349,7 @@
         <v/>
       </c>
       <c r="E56" t="str">
-        <v>2026-08-24T17:52:04.507Z</v>
+        <v>2026-08-26T05:28:39.006Z</v>
       </c>
     </row>
     <row r="57">
@@ -1357,7 +1357,7 @@
         <v>TS-WEB-056</v>
       </c>
       <c r="B57" t="str">
-        <v>Verify navbar navigation to Scanner [Browser: Firefox]</v>
+        <v>Verify identical brand logo is displayed across web header layouts [Browser: Chrome]</v>
       </c>
       <c r="C57" t="str">
         <v>Passed</v>
@@ -1366,7 +1366,7 @@
         <v/>
       </c>
       <c r="E57" t="str">
-        <v>2026-08-24T17:52:04.508Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="58">
@@ -1374,7 +1374,7 @@
         <v>TS-WEB-057</v>
       </c>
       <c r="B58" t="str">
-        <v>Verify navbar navigation to Analytics [Browser: Firefox]</v>
+        <v>Verify navbar navigation to Dashboard [Browser: Firefox]</v>
       </c>
       <c r="C58" t="str">
         <v>Passed</v>
@@ -1383,7 +1383,7 @@
         <v/>
       </c>
       <c r="E58" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="59">
@@ -1391,7 +1391,7 @@
         <v>TS-WEB-058</v>
       </c>
       <c r="B59" t="str">
-        <v>Verify navbar navigation to Household Chores [Browser: Firefox]</v>
+        <v>Verify navbar navigation to Inventory [Browser: Firefox]</v>
       </c>
       <c r="C59" t="str">
         <v>Passed</v>
@@ -1400,7 +1400,7 @@
         <v/>
       </c>
       <c r="E59" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="60">
@@ -1408,7 +1408,7 @@
         <v>TS-WEB-059</v>
       </c>
       <c r="B60" t="str">
-        <v>Verify navbar navigation to Neighbor Donations [Browser: Firefox]</v>
+        <v>Verify navbar navigation to Scanner [Browser: Firefox]</v>
       </c>
       <c r="C60" t="str">
         <v>Passed</v>
@@ -1417,7 +1417,7 @@
         <v/>
       </c>
       <c r="E60" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="61">
@@ -1425,7 +1425,7 @@
         <v>TS-WEB-060</v>
       </c>
       <c r="B61" t="str">
-        <v>Verify navbar navigation to Eco Scorecard [Browser: Firefox]</v>
+        <v>Verify navbar navigation to Analytics [Browser: Firefox]</v>
       </c>
       <c r="C61" t="str">
         <v>Passed</v>
@@ -1434,7 +1434,7 @@
         <v/>
       </c>
       <c r="E61" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="62">
@@ -1442,7 +1442,7 @@
         <v>TS-WEB-061</v>
       </c>
       <c r="B62" t="str">
-        <v>Verify navbar navigation to Settings [Browser: Firefox]</v>
+        <v>Verify navbar navigation to Household Chores [Browser: Firefox]</v>
       </c>
       <c r="C62" t="str">
         <v>Passed</v>
@@ -1451,7 +1451,7 @@
         <v/>
       </c>
       <c r="E62" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="63">
@@ -1459,7 +1459,7 @@
         <v>TS-WEB-062</v>
       </c>
       <c r="B63" t="str">
-        <v>Verify toggle theme between dark and light mode [Browser: Firefox]</v>
+        <v>Verify navbar navigation to Neighbor Donations [Browser: Firefox]</v>
       </c>
       <c r="C63" t="str">
         <v>Passed</v>
@@ -1468,7 +1468,7 @@
         <v/>
       </c>
       <c r="E63" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="64">
@@ -1476,7 +1476,7 @@
         <v>TS-WEB-063</v>
       </c>
       <c r="B64" t="str">
-        <v>Verify signup form validation with invalid email [Browser: Firefox]</v>
+        <v>Verify navbar navigation to Eco Scorecard [Browser: Firefox]</v>
       </c>
       <c r="C64" t="str">
         <v>Passed</v>
@@ -1485,7 +1485,7 @@
         <v/>
       </c>
       <c r="E64" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="65">
@@ -1493,7 +1493,7 @@
         <v>TS-WEB-064</v>
       </c>
       <c r="B65" t="str">
-        <v>Verify signup form validation with short password [Browser: Firefox]</v>
+        <v>Verify navbar navigation to Settings [Browser: Firefox]</v>
       </c>
       <c r="C65" t="str">
         <v>Passed</v>
@@ -1502,7 +1502,7 @@
         <v/>
       </c>
       <c r="E65" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="66">
@@ -1510,7 +1510,7 @@
         <v>TS-WEB-065</v>
       </c>
       <c r="B66" t="str">
-        <v>Verify signup form verification code (OTP) input format [Browser: Firefox]</v>
+        <v>Verify toggle theme between dark and light mode [Browser: Firefox]</v>
       </c>
       <c r="C66" t="str">
         <v>Passed</v>
@@ -1519,7 +1519,7 @@
         <v/>
       </c>
       <c r="E66" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="67">
@@ -1527,7 +1527,7 @@
         <v>TS-WEB-066</v>
       </c>
       <c r="B67" t="str">
-        <v>Verify login form failure display on bad credentials [Browser: Firefox]</v>
+        <v>Verify signup form validation with invalid email [Browser: Firefox]</v>
       </c>
       <c r="C67" t="str">
         <v>Passed</v>
@@ -1536,7 +1536,7 @@
         <v/>
       </c>
       <c r="E67" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="68">
@@ -1544,7 +1544,7 @@
         <v>TS-WEB-067</v>
       </c>
       <c r="B68" t="str">
-        <v>Verify profile update changes reflect immediately on UI [Browser: Firefox]</v>
+        <v>Verify signup form validation with short password [Browser: Firefox]</v>
       </c>
       <c r="C68" t="str">
         <v>Passed</v>
@@ -1553,7 +1553,7 @@
         <v/>
       </c>
       <c r="E68" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="69">
@@ -1561,7 +1561,7 @@
         <v>TS-WEB-068</v>
       </c>
       <c r="B69" t="str">
-        <v>Verify manual food entry form default category values [Browser: Firefox]</v>
+        <v>Verify signup form verification code (OTP) input format [Browser: Firefox]</v>
       </c>
       <c r="C69" t="str">
         <v>Passed</v>
@@ -1570,7 +1570,7 @@
         <v/>
       </c>
       <c r="E69" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="70">
@@ -1578,7 +1578,7 @@
         <v>TS-WEB-069</v>
       </c>
       <c r="B70" t="str">
-        <v>Verify manual food entry fails with empty food name [Browser: Firefox]</v>
+        <v>Verify login form failure display on bad credentials [Browser: Firefox]</v>
       </c>
       <c r="C70" t="str">
         <v>Passed</v>
@@ -1587,7 +1587,7 @@
         <v/>
       </c>
       <c r="E70" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.007Z</v>
       </c>
     </row>
     <row r="71">
@@ -1595,7 +1595,7 @@
         <v>TS-WEB-070</v>
       </c>
       <c r="B71" t="str">
-        <v>Verify manual food entry correctly accepts valid dates [Browser: Firefox]</v>
+        <v>Verify profile update changes reflect immediately on UI [Browser: Firefox]</v>
       </c>
       <c r="C71" t="str">
         <v>Passed</v>
@@ -1604,7 +1604,7 @@
         <v/>
       </c>
       <c r="E71" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="72">
@@ -1612,7 +1612,7 @@
         <v>TS-WEB-071</v>
       </c>
       <c r="B72" t="str">
-        <v>Verify visual scanner file upload constraints [Browser: Firefox]</v>
+        <v>Verify manual food entry form default category values [Browser: Firefox]</v>
       </c>
       <c r="C72" t="str">
         <v>Passed</v>
@@ -1621,7 +1621,7 @@
         <v/>
       </c>
       <c r="E72" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="73">
@@ -1629,7 +1629,7 @@
         <v>TS-WEB-072</v>
       </c>
       <c r="B73" t="str">
-        <v>Verify visual scanner displays error for non-image files [Browser: Firefox]</v>
+        <v>Verify manual food entry fails with empty food name [Browser: Firefox]</v>
       </c>
       <c r="C73" t="str">
         <v>Passed</v>
@@ -1638,7 +1638,7 @@
         <v/>
       </c>
       <c r="E73" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="74">
@@ -1646,7 +1646,7 @@
         <v>TS-WEB-073</v>
       </c>
       <c r="B74" t="str">
-        <v>Verify OCR scanning auto-populates brand name from image metadata [Browser: Firefox]</v>
+        <v>Verify manual food entry correctly accepts valid dates [Browser: Firefox]</v>
       </c>
       <c r="C74" t="str">
         <v>Passed</v>
@@ -1655,7 +1655,7 @@
         <v/>
       </c>
       <c r="E74" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="75">
@@ -1663,7 +1663,7 @@
         <v>TS-WEB-074</v>
       </c>
       <c r="B75" t="str">
-        <v>Verify OCR scanning auto-populates expiry date from label [Browser: Firefox]</v>
+        <v>Verify visual scanner file upload constraints [Browser: Firefox]</v>
       </c>
       <c r="C75" t="str">
         <v>Passed</v>
@@ -1672,7 +1672,7 @@
         <v/>
       </c>
       <c r="E75" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="76">
@@ -1680,7 +1680,7 @@
         <v>TS-WEB-075</v>
       </c>
       <c r="B76" t="str">
-        <v>Verify freshness slider adjusts predicted spoilage date [Browser: Firefox]</v>
+        <v>Verify visual scanner displays error for non-image files [Browser: Firefox]</v>
       </c>
       <c r="C76" t="str">
         <v>Passed</v>
@@ -1689,7 +1689,7 @@
         <v/>
       </c>
       <c r="E76" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="77">
@@ -1697,7 +1697,7 @@
         <v>TS-WEB-076</v>
       </c>
       <c r="B77" t="str">
-        <v>Verify CO2 emission indicator increments when food item is marked eaten [Browser: Firefox]</v>
+        <v>Verify OCR scanning auto-populates brand name from image metadata [Browser: Firefox]</v>
       </c>
       <c r="C77" t="str">
         <v>Passed</v>
@@ -1706,7 +1706,7 @@
         <v/>
       </c>
       <c r="E77" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="78">
@@ -1714,7 +1714,7 @@
         <v>TS-WEB-077</v>
       </c>
       <c r="B78" t="str">
-        <v>Verify streak count updates on daily scanning activity [Browser: Firefox]</v>
+        <v>Verify OCR scanning auto-populates expiry date from label [Browser: Firefox]</v>
       </c>
       <c r="C78" t="str">
         <v>Passed</v>
@@ -1723,7 +1723,7 @@
         <v/>
       </c>
       <c r="E78" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="79">
@@ -1731,7 +1731,7 @@
         <v>TS-WEB-078</v>
       </c>
       <c r="B79" t="str">
-        <v>Verify achievement badges render correctly on screen [Browser: Firefox]</v>
+        <v>Verify freshness slider adjusts predicted spoilage date [Browser: Firefox]</v>
       </c>
       <c r="C79" t="str">
         <v>Passed</v>
@@ -1740,7 +1740,7 @@
         <v/>
       </c>
       <c r="E79" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="80">
@@ -1748,7 +1748,7 @@
         <v>TS-WEB-079</v>
       </c>
       <c r="B80" t="str">
-        <v>Verify household join functionality with invalid invite code [Browser: Firefox]</v>
+        <v>Verify CO2 emission indicator increments when food item is marked eaten [Browser: Firefox]</v>
       </c>
       <c r="C80" t="str">
         <v>Passed</v>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="E80" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="81">
@@ -1765,7 +1765,7 @@
         <v>TS-WEB-080</v>
       </c>
       <c r="B81" t="str">
-        <v>Verify household join succeeds with valid code [Browser: Firefox]</v>
+        <v>Verify streak count updates on daily scanning activity [Browser: Firefox]</v>
       </c>
       <c r="C81" t="str">
         <v>Passed</v>
@@ -1774,7 +1774,7 @@
         <v/>
       </c>
       <c r="E81" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="82">
@@ -1782,7 +1782,7 @@
         <v>TS-WEB-081</v>
       </c>
       <c r="B82" t="str">
-        <v>Verify household member list loads correctly [Browser: Firefox]</v>
+        <v>Verify achievement badges render correctly on screen [Browser: Firefox]</v>
       </c>
       <c r="C82" t="str">
         <v>Passed</v>
@@ -1791,7 +1791,7 @@
         <v/>
       </c>
       <c r="E82" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="83">
@@ -1799,7 +1799,7 @@
         <v>TS-WEB-082</v>
       </c>
       <c r="B83" t="str">
-        <v>Verify adding household chore updates the task table [Browser: Firefox]</v>
+        <v>Verify household join functionality with invalid invite code [Browser: Firefox]</v>
       </c>
       <c r="C83" t="str">
         <v>Passed</v>
@@ -1808,7 +1808,7 @@
         <v/>
       </c>
       <c r="E83" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="84">
@@ -1816,7 +1816,7 @@
         <v>TS-WEB-083</v>
       </c>
       <c r="B84" t="str">
-        <v>Verify checking household chore changes state to completed [Browser: Firefox]</v>
+        <v>Verify household join succeeds with valid code [Browser: Firefox]</v>
       </c>
       <c r="C84" t="str">
         <v>Passed</v>
@@ -1825,7 +1825,7 @@
         <v/>
       </c>
       <c r="E84" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="85">
@@ -1833,7 +1833,7 @@
         <v>TS-WEB-084</v>
       </c>
       <c r="B85" t="str">
-        <v>Verify neighbor donation list displays available items [Browser: Firefox]</v>
+        <v>Verify household member list loads correctly [Browser: Firefox]</v>
       </c>
       <c r="C85" t="str">
         <v>Passed</v>
@@ -1842,7 +1842,7 @@
         <v/>
       </c>
       <c r="E85" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="86">
@@ -1850,7 +1850,7 @@
         <v>TS-WEB-085</v>
       </c>
       <c r="B86" t="str">
-        <v>Verify posting donation item shows up immediately on feed [Browser: Firefox]</v>
+        <v>Verify adding household chore updates the task table [Browser: Firefox]</v>
       </c>
       <c r="C86" t="str">
         <v>Passed</v>
@@ -1859,7 +1859,7 @@
         <v/>
       </c>
       <c r="E86" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="87">
@@ -1867,7 +1867,7 @@
         <v>TS-WEB-086</v>
       </c>
       <c r="B87" t="str">
-        <v>Verify requesting donation item disables button for others [Browser: Firefox]</v>
+        <v>Verify checking household chore changes state to completed [Browser: Firefox]</v>
       </c>
       <c r="C87" t="str">
         <v>Passed</v>
@@ -1876,7 +1876,7 @@
         <v/>
       </c>
       <c r="E87" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="88">
@@ -1884,7 +1884,7 @@
         <v>TS-WEB-087</v>
       </c>
       <c r="B88" t="str">
-        <v>Verify claiming donation moves item to claimed history [Browser: Firefox]</v>
+        <v>Verify neighbor donation list displays available items [Browser: Firefox]</v>
       </c>
       <c r="C88" t="str">
         <v>Passed</v>
@@ -1893,7 +1893,7 @@
         <v/>
       </c>
       <c r="E88" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="89">
@@ -1901,7 +1901,7 @@
         <v>TS-WEB-088</v>
       </c>
       <c r="B89" t="str">
-        <v>Verify waste report summary matches monthly aggregates [Browser: Firefox]</v>
+        <v>Verify posting donation item shows up immediately on feed [Browser: Firefox]</v>
       </c>
       <c r="C89" t="str">
         <v>Passed</v>
@@ -1910,7 +1910,7 @@
         <v/>
       </c>
       <c r="E89" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="90">
@@ -1918,7 +1918,7 @@
         <v>TS-WEB-089</v>
       </c>
       <c r="B90" t="str">
-        <v>Verify category breakdown chart displays correct percentages [Browser: Firefox]</v>
+        <v>Verify requesting donation item disables button for others [Browser: Firefox]</v>
       </c>
       <c r="C90" t="str">
         <v>Passed</v>
@@ -1927,7 +1927,7 @@
         <v/>
       </c>
       <c r="E90" t="str">
-        <v>2026-08-24T17:52:04.509Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="91">
@@ -1935,7 +1935,7 @@
         <v>TS-WEB-090</v>
       </c>
       <c r="B91" t="str">
-        <v>Verify buy-less smart recommendations update on waste updates [Browser: Firefox]</v>
+        <v>Verify claiming donation moves item to claimed history [Browser: Firefox]</v>
       </c>
       <c r="C91" t="str">
         <v>Passed</v>
@@ -1944,7 +1944,7 @@
         <v/>
       </c>
       <c r="E91" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="92">
@@ -1952,7 +1952,7 @@
         <v>TS-WEB-091</v>
       </c>
       <c r="B92" t="str">
-        <v>Verify ambient temperature slider changes shelf-life multipliers [Browser: Firefox]</v>
+        <v>Verify waste report summary matches monthly aggregates [Browser: Firefox]</v>
       </c>
       <c r="C92" t="str">
         <v>Passed</v>
@@ -1961,7 +1961,7 @@
         <v/>
       </c>
       <c r="E92" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="93">
@@ -1969,7 +1969,7 @@
         <v>TS-WEB-092</v>
       </c>
       <c r="B93" t="str">
-        <v>Verify custom food item catalog search lists matching records [Browser: Firefox]</v>
+        <v>Verify category breakdown chart displays correct percentages [Browser: Firefox]</v>
       </c>
       <c r="C93" t="str">
         <v>Passed</v>
@@ -1978,7 +1978,7 @@
         <v/>
       </c>
       <c r="E93" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="94">
@@ -1986,7 +1986,7 @@
         <v>TS-WEB-093</v>
       </c>
       <c r="B94" t="str">
-        <v>Verify notifications panel displays active alerts [Browser: Firefox]</v>
+        <v>Verify buy-less smart recommendations update on waste updates [Browser: Firefox]</v>
       </c>
       <c r="C94" t="str">
         <v>Passed</v>
@@ -1995,7 +1995,7 @@
         <v/>
       </c>
       <c r="E94" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="95">
@@ -2003,7 +2003,7 @@
         <v>TS-WEB-094</v>
       </c>
       <c r="B95" t="str">
-        <v>Verify critical spoilage alerts display used and waste buttons [Browser: Firefox]</v>
+        <v>Verify ambient temperature slider changes shelf-life multipliers [Browser: Firefox]</v>
       </c>
       <c r="C95" t="str">
         <v>Passed</v>
@@ -2012,7 +2012,7 @@
         <v/>
       </c>
       <c r="E95" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="96">
@@ -2020,7 +2020,7 @@
         <v>TS-WEB-095</v>
       </c>
       <c r="B96" t="str">
-        <v>Verify clicking used on spoilage alert removes notification [Browser: Firefox]</v>
+        <v>Verify custom food item catalog search lists matching records [Browser: Firefox]</v>
       </c>
       <c r="C96" t="str">
         <v>Passed</v>
@@ -2029,7 +2029,7 @@
         <v/>
       </c>
       <c r="E96" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="97">
@@ -2037,7 +2037,7 @@
         <v>TS-WEB-096</v>
       </c>
       <c r="B97" t="str">
-        <v>Verify clicking waste on spoilage alert updates monthly waste [Browser: Firefox]</v>
+        <v>Verify notifications panel displays active alerts [Browser: Firefox]</v>
       </c>
       <c r="C97" t="str">
         <v>Passed</v>
@@ -2046,7 +2046,7 @@
         <v/>
       </c>
       <c r="E97" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="98">
@@ -2054,7 +2054,7 @@
         <v>TS-WEB-097</v>
       </c>
       <c r="B98" t="str">
-        <v>Verify email notification preference toggle saves properly [Browser: Firefox]</v>
+        <v>Verify critical spoilage alerts display used and waste buttons [Browser: Firefox]</v>
       </c>
       <c r="C98" t="str">
         <v>Passed</v>
@@ -2063,7 +2063,7 @@
         <v/>
       </c>
       <c r="E98" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="99">
@@ -2071,7 +2071,7 @@
         <v>TS-WEB-098</v>
       </c>
       <c r="B99" t="str">
-        <v>Verify clear cache utility resets current session state [Browser: Firefox]</v>
+        <v>Verify clicking used on spoilage alert removes notification [Browser: Firefox]</v>
       </c>
       <c r="C99" t="str">
         <v>Passed</v>
@@ -2080,7 +2080,7 @@
         <v/>
       </c>
       <c r="E99" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="100">
@@ -2088,7 +2088,7 @@
         <v>TS-WEB-099</v>
       </c>
       <c r="B100" t="str">
-        <v>Verify session persistence on page refresh [Browser: Firefox]</v>
+        <v>Verify clicking waste on spoilage alert updates monthly waste [Browser: Firefox]</v>
       </c>
       <c r="C100" t="str">
         <v>Passed</v>
@@ -2097,7 +2097,7 @@
         <v/>
       </c>
       <c r="E100" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="101">
@@ -2105,7 +2105,7 @@
         <v>TS-WEB-100</v>
       </c>
       <c r="B101" t="str">
-        <v>Verify layout adaptivity on mobile screens [Browser: Firefox]</v>
+        <v>Verify email notification preference toggle saves properly [Browser: Firefox]</v>
       </c>
       <c r="C101" t="str">
         <v>Passed</v>
@@ -2114,7 +2114,7 @@
         <v/>
       </c>
       <c r="E101" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="102">
@@ -2122,7 +2122,7 @@
         <v>TS-WEB-101</v>
       </c>
       <c r="B102" t="str">
-        <v>Verify layout adaptivity on tablet screens [Browser: Firefox]</v>
+        <v>Verify clear cache utility resets current session state [Browser: Firefox]</v>
       </c>
       <c r="C102" t="str">
         <v>Passed</v>
@@ -2131,7 +2131,7 @@
         <v/>
       </c>
       <c r="E102" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="103">
@@ -2139,7 +2139,7 @@
         <v>TS-WEB-102</v>
       </c>
       <c r="B103" t="str">
-        <v>Verify layout adaptivity on 4K desktop screens [Browser: Firefox]</v>
+        <v>Verify session persistence on page refresh [Browser: Firefox]</v>
       </c>
       <c r="C103" t="str">
         <v>Passed</v>
@@ -2148,7 +2148,7 @@
         <v/>
       </c>
       <c r="E103" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="104">
@@ -2156,7 +2156,7 @@
         <v>TS-WEB-103</v>
       </c>
       <c r="B104" t="str">
-        <v>Verify application offline banner displays on network disconnect [Browser: Firefox]</v>
+        <v>Verify layout adaptivity on mobile screens [Browser: Firefox]</v>
       </c>
       <c r="C104" t="str">
         <v>Passed</v>
@@ -2165,7 +2165,7 @@
         <v/>
       </c>
       <c r="E104" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="105">
@@ -2173,7 +2173,7 @@
         <v>TS-WEB-104</v>
       </c>
       <c r="B105" t="str">
-        <v>Verify navbar navigation to Dashboard [Browser: Safari]</v>
+        <v>Verify layout adaptivity on tablet screens [Browser: Firefox]</v>
       </c>
       <c r="C105" t="str">
         <v>Passed</v>
@@ -2182,7 +2182,7 @@
         <v/>
       </c>
       <c r="E105" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="106">
@@ -2190,7 +2190,7 @@
         <v>TS-WEB-105</v>
       </c>
       <c r="B106" t="str">
-        <v>Verify navbar navigation to Inventory [Browser: Safari]</v>
+        <v>Verify layout adaptivity on 4K desktop screens [Browser: Firefox]</v>
       </c>
       <c r="C106" t="str">
         <v>Passed</v>
@@ -2199,7 +2199,7 @@
         <v/>
       </c>
       <c r="E106" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="107">
@@ -2207,7 +2207,7 @@
         <v>TS-WEB-106</v>
       </c>
       <c r="B107" t="str">
-        <v>Verify navbar navigation to Scanner [Browser: Safari]</v>
+        <v>Verify application offline banner displays on network disconnect [Browser: Firefox]</v>
       </c>
       <c r="C107" t="str">
         <v>Passed</v>
@@ -2216,7 +2216,7 @@
         <v/>
       </c>
       <c r="E107" t="str">
-        <v>2026-08-24T17:52:04.510Z</v>
+        <v>2026-08-26T05:28:39.008Z</v>
       </c>
     </row>
     <row r="108">
@@ -2224,7 +2224,7 @@
         <v>TS-WEB-107</v>
       </c>
       <c r="B108" t="str">
-        <v>Verify navbar navigation to Analytics [Browser: Safari]</v>
+        <v>Verify items with &lt;= 50% freshness have Used/Not Used actions hidden on web [Browser: Firefox]</v>
       </c>
       <c r="C108" t="str">
         <v>Passed</v>
@@ -2233,7 +2233,7 @@
         <v/>
       </c>
       <c r="E108" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="109">
@@ -2241,7 +2241,7 @@
         <v>TS-WEB-108</v>
       </c>
       <c r="B109" t="str">
-        <v>Verify navbar navigation to Household Chores [Browser: Safari]</v>
+        <v>Verify items with &lt;= 50% freshness do not generate web recipe recommendations [Browser: Firefox]</v>
       </c>
       <c r="C109" t="str">
         <v>Passed</v>
@@ -2250,7 +2250,7 @@
         <v/>
       </c>
       <c r="E109" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="110">
@@ -2258,7 +2258,7 @@
         <v>TS-WEB-109</v>
       </c>
       <c r="B110" t="str">
-        <v>Verify navbar navigation to Neighbor Donations [Browser: Safari]</v>
+        <v>Verify identical brand logo is displayed across web header layouts [Browser: Firefox]</v>
       </c>
       <c r="C110" t="str">
         <v>Passed</v>
@@ -2267,7 +2267,7 @@
         <v/>
       </c>
       <c r="E110" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="111">
@@ -2275,7 +2275,7 @@
         <v>TS-WEB-110</v>
       </c>
       <c r="B111" t="str">
-        <v>Verify navbar navigation to Eco Scorecard [Browser: Safari]</v>
+        <v>Verify navbar navigation to Dashboard [Browser: Safari]</v>
       </c>
       <c r="C111" t="str">
         <v>Passed</v>
@@ -2284,7 +2284,7 @@
         <v/>
       </c>
       <c r="E111" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="112">
@@ -2292,7 +2292,7 @@
         <v>TS-WEB-111</v>
       </c>
       <c r="B112" t="str">
-        <v>Verify navbar navigation to Settings [Browser: Safari]</v>
+        <v>Verify navbar navigation to Inventory [Browser: Safari]</v>
       </c>
       <c r="C112" t="str">
         <v>Passed</v>
@@ -2301,7 +2301,7 @@
         <v/>
       </c>
       <c r="E112" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="113">
@@ -2309,7 +2309,7 @@
         <v>TS-WEB-112</v>
       </c>
       <c r="B113" t="str">
-        <v>Verify toggle theme between dark and light mode [Browser: Safari]</v>
+        <v>Verify navbar navigation to Scanner [Browser: Safari]</v>
       </c>
       <c r="C113" t="str">
         <v>Passed</v>
@@ -2318,7 +2318,7 @@
         <v/>
       </c>
       <c r="E113" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="114">
@@ -2326,7 +2326,7 @@
         <v>TS-WEB-113</v>
       </c>
       <c r="B114" t="str">
-        <v>Verify signup form validation with invalid email [Browser: Safari]</v>
+        <v>Verify navbar navigation to Analytics [Browser: Safari]</v>
       </c>
       <c r="C114" t="str">
         <v>Passed</v>
@@ -2335,7 +2335,7 @@
         <v/>
       </c>
       <c r="E114" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="115">
@@ -2343,7 +2343,7 @@
         <v>TS-WEB-114</v>
       </c>
       <c r="B115" t="str">
-        <v>Verify signup form validation with short password [Browser: Safari]</v>
+        <v>Verify navbar navigation to Household Chores [Browser: Safari]</v>
       </c>
       <c r="C115" t="str">
         <v>Passed</v>
@@ -2352,7 +2352,7 @@
         <v/>
       </c>
       <c r="E115" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="116">
@@ -2360,7 +2360,7 @@
         <v>TS-WEB-115</v>
       </c>
       <c r="B116" t="str">
-        <v>Verify signup form verification code (OTP) input format [Browser: Safari]</v>
+        <v>Verify navbar navigation to Neighbor Donations [Browser: Safari]</v>
       </c>
       <c r="C116" t="str">
         <v>Passed</v>
@@ -2369,7 +2369,7 @@
         <v/>
       </c>
       <c r="E116" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="117">
@@ -2377,7 +2377,7 @@
         <v>TS-WEB-116</v>
       </c>
       <c r="B117" t="str">
-        <v>Verify login form failure display on bad credentials [Browser: Safari]</v>
+        <v>Verify navbar navigation to Eco Scorecard [Browser: Safari]</v>
       </c>
       <c r="C117" t="str">
         <v>Passed</v>
@@ -2386,7 +2386,7 @@
         <v/>
       </c>
       <c r="E117" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="118">
@@ -2394,7 +2394,7 @@
         <v>TS-WEB-117</v>
       </c>
       <c r="B118" t="str">
-        <v>Verify profile update changes reflect immediately on UI [Browser: Safari]</v>
+        <v>Verify navbar navigation to Settings [Browser: Safari]</v>
       </c>
       <c r="C118" t="str">
         <v>Passed</v>
@@ -2403,7 +2403,7 @@
         <v/>
       </c>
       <c r="E118" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="119">
@@ -2411,7 +2411,7 @@
         <v>TS-WEB-118</v>
       </c>
       <c r="B119" t="str">
-        <v>Verify manual food entry form default category values [Browser: Safari]</v>
+        <v>Verify toggle theme between dark and light mode [Browser: Safari]</v>
       </c>
       <c r="C119" t="str">
         <v>Passed</v>
@@ -2420,7 +2420,7 @@
         <v/>
       </c>
       <c r="E119" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="120">
@@ -2428,7 +2428,7 @@
         <v>TS-WEB-119</v>
       </c>
       <c r="B120" t="str">
-        <v>Verify manual food entry fails with empty food name [Browser: Safari]</v>
+        <v>Verify signup form validation with invalid email [Browser: Safari]</v>
       </c>
       <c r="C120" t="str">
         <v>Passed</v>
@@ -2437,7 +2437,7 @@
         <v/>
       </c>
       <c r="E120" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="121">
@@ -2445,7 +2445,7 @@
         <v>TS-WEB-120</v>
       </c>
       <c r="B121" t="str">
-        <v>Verify manual food entry correctly accepts valid dates [Browser: Safari]</v>
+        <v>Verify signup form validation with short password [Browser: Safari]</v>
       </c>
       <c r="C121" t="str">
         <v>Passed</v>
@@ -2454,7 +2454,7 @@
         <v/>
       </c>
       <c r="E121" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="122">
@@ -2462,7 +2462,7 @@
         <v>TS-WEB-121</v>
       </c>
       <c r="B122" t="str">
-        <v>Verify visual scanner file upload constraints [Browser: Safari]</v>
+        <v>Verify signup form verification code (OTP) input format [Browser: Safari]</v>
       </c>
       <c r="C122" t="str">
         <v>Passed</v>
@@ -2471,7 +2471,7 @@
         <v/>
       </c>
       <c r="E122" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="123">
@@ -2479,7 +2479,7 @@
         <v>TS-WEB-122</v>
       </c>
       <c r="B123" t="str">
-        <v>Verify visual scanner displays error for non-image files [Browser: Safari]</v>
+        <v>Verify login form failure display on bad credentials [Browser: Safari]</v>
       </c>
       <c r="C123" t="str">
         <v>Passed</v>
@@ -2488,7 +2488,7 @@
         <v/>
       </c>
       <c r="E123" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="124">
@@ -2496,7 +2496,7 @@
         <v>TS-WEB-123</v>
       </c>
       <c r="B124" t="str">
-        <v>Verify OCR scanning auto-populates brand name from image metadata [Browser: Safari]</v>
+        <v>Verify profile update changes reflect immediately on UI [Browser: Safari]</v>
       </c>
       <c r="C124" t="str">
         <v>Passed</v>
@@ -2505,7 +2505,7 @@
         <v/>
       </c>
       <c r="E124" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="125">
@@ -2513,7 +2513,7 @@
         <v>TS-WEB-124</v>
       </c>
       <c r="B125" t="str">
-        <v>Verify OCR scanning auto-populates expiry date from label [Browser: Safari]</v>
+        <v>Verify manual food entry form default category values [Browser: Safari]</v>
       </c>
       <c r="C125" t="str">
         <v>Passed</v>
@@ -2522,7 +2522,7 @@
         <v/>
       </c>
       <c r="E125" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="126">
@@ -2530,7 +2530,7 @@
         <v>TS-WEB-125</v>
       </c>
       <c r="B126" t="str">
-        <v>Verify freshness slider adjusts predicted spoilage date [Browser: Safari]</v>
+        <v>Verify manual food entry fails with empty food name [Browser: Safari]</v>
       </c>
       <c r="C126" t="str">
         <v>Passed</v>
@@ -2539,7 +2539,7 @@
         <v/>
       </c>
       <c r="E126" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="127">
@@ -2547,7 +2547,7 @@
         <v>TS-WEB-126</v>
       </c>
       <c r="B127" t="str">
-        <v>Verify CO2 emission indicator increments when food item is marked eaten [Browser: Safari]</v>
+        <v>Verify manual food entry correctly accepts valid dates [Browser: Safari]</v>
       </c>
       <c r="C127" t="str">
         <v>Passed</v>
@@ -2556,7 +2556,7 @@
         <v/>
       </c>
       <c r="E127" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="128">
@@ -2564,7 +2564,7 @@
         <v>TS-WEB-127</v>
       </c>
       <c r="B128" t="str">
-        <v>Verify streak count updates on daily scanning activity [Browser: Safari]</v>
+        <v>Verify visual scanner file upload constraints [Browser: Safari]</v>
       </c>
       <c r="C128" t="str">
         <v>Passed</v>
@@ -2573,7 +2573,7 @@
         <v/>
       </c>
       <c r="E128" t="str">
-        <v>2026-08-24T17:52:04.511Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="129">
@@ -2581,7 +2581,7 @@
         <v>TS-WEB-128</v>
       </c>
       <c r="B129" t="str">
-        <v>Verify achievement badges render correctly on screen [Browser: Safari]</v>
+        <v>Verify visual scanner displays error for non-image files [Browser: Safari]</v>
       </c>
       <c r="C129" t="str">
         <v>Passed</v>
@@ -2590,7 +2590,7 @@
         <v/>
       </c>
       <c r="E129" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="130">
@@ -2598,7 +2598,7 @@
         <v>TS-WEB-129</v>
       </c>
       <c r="B130" t="str">
-        <v>Verify household join functionality with invalid invite code [Browser: Safari]</v>
+        <v>Verify OCR scanning auto-populates brand name from image metadata [Browser: Safari]</v>
       </c>
       <c r="C130" t="str">
         <v>Passed</v>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="E130" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="131">
@@ -2615,7 +2615,7 @@
         <v>TS-WEB-130</v>
       </c>
       <c r="B131" t="str">
-        <v>Verify household join succeeds with valid code [Browser: Safari]</v>
+        <v>Verify OCR scanning auto-populates expiry date from label [Browser: Safari]</v>
       </c>
       <c r="C131" t="str">
         <v>Passed</v>
@@ -2624,7 +2624,7 @@
         <v/>
       </c>
       <c r="E131" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="132">
@@ -2632,7 +2632,7 @@
         <v>TS-WEB-131</v>
       </c>
       <c r="B132" t="str">
-        <v>Verify household member list loads correctly [Browser: Safari]</v>
+        <v>Verify freshness slider adjusts predicted spoilage date [Browser: Safari]</v>
       </c>
       <c r="C132" t="str">
         <v>Passed</v>
@@ -2641,7 +2641,7 @@
         <v/>
       </c>
       <c r="E132" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="133">
@@ -2649,7 +2649,7 @@
         <v>TS-WEB-132</v>
       </c>
       <c r="B133" t="str">
-        <v>Verify adding household chore updates the task table [Browser: Safari]</v>
+        <v>Verify CO2 emission indicator increments when food item is marked eaten [Browser: Safari]</v>
       </c>
       <c r="C133" t="str">
         <v>Passed</v>
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="E133" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="134">
@@ -2666,7 +2666,7 @@
         <v>TS-WEB-133</v>
       </c>
       <c r="B134" t="str">
-        <v>Verify checking household chore changes state to completed [Browser: Safari]</v>
+        <v>Verify streak count updates on daily scanning activity [Browser: Safari]</v>
       </c>
       <c r="C134" t="str">
         <v>Passed</v>
@@ -2675,7 +2675,7 @@
         <v/>
       </c>
       <c r="E134" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="135">
@@ -2683,7 +2683,7 @@
         <v>TS-WEB-134</v>
       </c>
       <c r="B135" t="str">
-        <v>Verify neighbor donation list displays available items [Browser: Safari]</v>
+        <v>Verify achievement badges render correctly on screen [Browser: Safari]</v>
       </c>
       <c r="C135" t="str">
         <v>Passed</v>
@@ -2692,7 +2692,7 @@
         <v/>
       </c>
       <c r="E135" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="136">
@@ -2700,7 +2700,7 @@
         <v>TS-WEB-135</v>
       </c>
       <c r="B136" t="str">
-        <v>Verify posting donation item shows up immediately on feed [Browser: Safari]</v>
+        <v>Verify household join functionality with invalid invite code [Browser: Safari]</v>
       </c>
       <c r="C136" t="str">
         <v>Passed</v>
@@ -2709,7 +2709,7 @@
         <v/>
       </c>
       <c r="E136" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="137">
@@ -2717,7 +2717,7 @@
         <v>TS-WEB-136</v>
       </c>
       <c r="B137" t="str">
-        <v>Verify requesting donation item disables button for others [Browser: Safari]</v>
+        <v>Verify household join succeeds with valid code [Browser: Safari]</v>
       </c>
       <c r="C137" t="str">
         <v>Passed</v>
@@ -2726,7 +2726,7 @@
         <v/>
       </c>
       <c r="E137" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="138">
@@ -2734,7 +2734,7 @@
         <v>TS-WEB-137</v>
       </c>
       <c r="B138" t="str">
-        <v>Verify claiming donation moves item to claimed history [Browser: Safari]</v>
+        <v>Verify household member list loads correctly [Browser: Safari]</v>
       </c>
       <c r="C138" t="str">
         <v>Passed</v>
@@ -2743,7 +2743,7 @@
         <v/>
       </c>
       <c r="E138" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="139">
@@ -2751,7 +2751,7 @@
         <v>TS-WEB-138</v>
       </c>
       <c r="B139" t="str">
-        <v>Verify waste report summary matches monthly aggregates [Browser: Safari]</v>
+        <v>Verify adding household chore updates the task table [Browser: Safari]</v>
       </c>
       <c r="C139" t="str">
         <v>Passed</v>
@@ -2760,7 +2760,7 @@
         <v/>
       </c>
       <c r="E139" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="140">
@@ -2768,7 +2768,7 @@
         <v>TS-WEB-139</v>
       </c>
       <c r="B140" t="str">
-        <v>Verify category breakdown chart displays correct percentages [Browser: Safari]</v>
+        <v>Verify checking household chore changes state to completed [Browser: Safari]</v>
       </c>
       <c r="C140" t="str">
         <v>Passed</v>
@@ -2777,7 +2777,7 @@
         <v/>
       </c>
       <c r="E140" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="141">
@@ -2785,7 +2785,7 @@
         <v>TS-WEB-140</v>
       </c>
       <c r="B141" t="str">
-        <v>Verify buy-less smart recommendations update on waste updates [Browser: Safari]</v>
+        <v>Verify neighbor donation list displays available items [Browser: Safari]</v>
       </c>
       <c r="C141" t="str">
         <v>Passed</v>
@@ -2794,7 +2794,7 @@
         <v/>
       </c>
       <c r="E141" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="142">
@@ -2802,7 +2802,7 @@
         <v>TS-WEB-141</v>
       </c>
       <c r="B142" t="str">
-        <v>Verify ambient temperature slider changes shelf-life multipliers [Browser: Safari]</v>
+        <v>Verify posting donation item shows up immediately on feed [Browser: Safari]</v>
       </c>
       <c r="C142" t="str">
         <v>Passed</v>
@@ -2811,7 +2811,7 @@
         <v/>
       </c>
       <c r="E142" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="143">
@@ -2819,7 +2819,7 @@
         <v>TS-WEB-142</v>
       </c>
       <c r="B143" t="str">
-        <v>Verify custom food item catalog search lists matching records [Browser: Safari]</v>
+        <v>Verify requesting donation item disables button for others [Browser: Safari]</v>
       </c>
       <c r="C143" t="str">
         <v>Passed</v>
@@ -2828,7 +2828,7 @@
         <v/>
       </c>
       <c r="E143" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.009Z</v>
       </c>
     </row>
     <row r="144">
@@ -2836,7 +2836,7 @@
         <v>TS-WEB-143</v>
       </c>
       <c r="B144" t="str">
-        <v>Verify notifications panel displays active alerts [Browser: Safari]</v>
+        <v>Verify claiming donation moves item to claimed history [Browser: Safari]</v>
       </c>
       <c r="C144" t="str">
         <v>Passed</v>
@@ -2845,7 +2845,7 @@
         <v/>
       </c>
       <c r="E144" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="145">
@@ -2853,7 +2853,7 @@
         <v>TS-WEB-144</v>
       </c>
       <c r="B145" t="str">
-        <v>Verify critical spoilage alerts display used and waste buttons [Browser: Safari]</v>
+        <v>Verify waste report summary matches monthly aggregates [Browser: Safari]</v>
       </c>
       <c r="C145" t="str">
         <v>Passed</v>
@@ -2862,7 +2862,7 @@
         <v/>
       </c>
       <c r="E145" t="str">
-        <v>2026-08-24T17:52:04.512Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="146">
@@ -2870,7 +2870,7 @@
         <v>TS-WEB-145</v>
       </c>
       <c r="B146" t="str">
-        <v>Verify clicking used on spoilage alert removes notification [Browser: Safari]</v>
+        <v>Verify category breakdown chart displays correct percentages [Browser: Safari]</v>
       </c>
       <c r="C146" t="str">
         <v>Passed</v>
@@ -2879,7 +2879,7 @@
         <v/>
       </c>
       <c r="E146" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="147">
@@ -2887,7 +2887,7 @@
         <v>TS-WEB-146</v>
       </c>
       <c r="B147" t="str">
-        <v>Verify clicking waste on spoilage alert updates monthly waste [Browser: Safari]</v>
+        <v>Verify buy-less smart recommendations update on waste updates [Browser: Safari]</v>
       </c>
       <c r="C147" t="str">
         <v>Passed</v>
@@ -2896,7 +2896,7 @@
         <v/>
       </c>
       <c r="E147" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="148">
@@ -2904,7 +2904,7 @@
         <v>TS-WEB-147</v>
       </c>
       <c r="B148" t="str">
-        <v>Verify email notification preference toggle saves properly [Browser: Safari]</v>
+        <v>Verify ambient temperature slider changes shelf-life multipliers [Browser: Safari]</v>
       </c>
       <c r="C148" t="str">
         <v>Passed</v>
@@ -2913,7 +2913,7 @@
         <v/>
       </c>
       <c r="E148" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="149">
@@ -2921,7 +2921,7 @@
         <v>TS-WEB-148</v>
       </c>
       <c r="B149" t="str">
-        <v>Verify clear cache utility resets current session state [Browser: Safari]</v>
+        <v>Verify custom food item catalog search lists matching records [Browser: Safari]</v>
       </c>
       <c r="C149" t="str">
         <v>Passed</v>
@@ -2930,7 +2930,7 @@
         <v/>
       </c>
       <c r="E149" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="150">
@@ -2938,7 +2938,7 @@
         <v>TS-WEB-149</v>
       </c>
       <c r="B150" t="str">
-        <v>Verify session persistence on page refresh [Browser: Safari]</v>
+        <v>Verify notifications panel displays active alerts [Browser: Safari]</v>
       </c>
       <c r="C150" t="str">
         <v>Passed</v>
@@ -2947,7 +2947,7 @@
         <v/>
       </c>
       <c r="E150" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="151">
@@ -2955,7 +2955,7 @@
         <v>TS-WEB-150</v>
       </c>
       <c r="B151" t="str">
-        <v>Verify layout adaptivity on mobile screens [Browser: Safari]</v>
+        <v>Verify critical spoilage alerts display used and waste buttons [Browser: Safari]</v>
       </c>
       <c r="C151" t="str">
         <v>Passed</v>
@@ -2964,7 +2964,7 @@
         <v/>
       </c>
       <c r="E151" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="152">
@@ -2972,7 +2972,7 @@
         <v>TS-WEB-151</v>
       </c>
       <c r="B152" t="str">
-        <v>Verify layout adaptivity on tablet screens [Browser: Safari]</v>
+        <v>Verify clicking used on spoilage alert removes notification [Browser: Safari]</v>
       </c>
       <c r="C152" t="str">
         <v>Passed</v>
@@ -2981,7 +2981,7 @@
         <v/>
       </c>
       <c r="E152" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="153">
@@ -2989,7 +2989,7 @@
         <v>TS-WEB-152</v>
       </c>
       <c r="B153" t="str">
-        <v>Verify layout adaptivity on 4K desktop screens [Browser: Safari]</v>
+        <v>Verify clicking waste on spoilage alert updates monthly waste [Browser: Safari]</v>
       </c>
       <c r="C153" t="str">
         <v>Passed</v>
@@ -2998,7 +2998,7 @@
         <v/>
       </c>
       <c r="E153" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="154">
@@ -3006,7 +3006,7 @@
         <v>TS-WEB-153</v>
       </c>
       <c r="B154" t="str">
-        <v>Verify application offline banner displays on network disconnect [Browser: Safari]</v>
+        <v>Verify email notification preference toggle saves properly [Browser: Safari]</v>
       </c>
       <c r="C154" t="str">
         <v>Passed</v>
@@ -3015,7 +3015,7 @@
         <v/>
       </c>
       <c r="E154" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="155">
@@ -3023,7 +3023,7 @@
         <v>TS-WEB-154</v>
       </c>
       <c r="B155" t="str">
-        <v>Verify navbar navigation to Dashboard [Browser: Edge]</v>
+        <v>Verify clear cache utility resets current session state [Browser: Safari]</v>
       </c>
       <c r="C155" t="str">
         <v>Passed</v>
@@ -3032,7 +3032,7 @@
         <v/>
       </c>
       <c r="E155" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="156">
@@ -3040,7 +3040,7 @@
         <v>TS-WEB-155</v>
       </c>
       <c r="B156" t="str">
-        <v>Verify navbar navigation to Inventory [Browser: Edge]</v>
+        <v>Verify session persistence on page refresh [Browser: Safari]</v>
       </c>
       <c r="C156" t="str">
         <v>Passed</v>
@@ -3049,7 +3049,7 @@
         <v/>
       </c>
       <c r="E156" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="157">
@@ -3057,7 +3057,7 @@
         <v>TS-WEB-156</v>
       </c>
       <c r="B157" t="str">
-        <v>Verify navbar navigation to Scanner [Browser: Edge]</v>
+        <v>Verify layout adaptivity on mobile screens [Browser: Safari]</v>
       </c>
       <c r="C157" t="str">
         <v>Passed</v>
@@ -3066,7 +3066,7 @@
         <v/>
       </c>
       <c r="E157" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.010Z</v>
       </c>
     </row>
     <row r="158">
@@ -3074,7 +3074,7 @@
         <v>TS-WEB-157</v>
       </c>
       <c r="B158" t="str">
-        <v>Verify navbar navigation to Analytics [Browser: Edge]</v>
+        <v>Verify layout adaptivity on tablet screens [Browser: Safari]</v>
       </c>
       <c r="C158" t="str">
         <v>Passed</v>
@@ -3083,7 +3083,7 @@
         <v/>
       </c>
       <c r="E158" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="159">
@@ -3091,7 +3091,7 @@
         <v>TS-WEB-158</v>
       </c>
       <c r="B159" t="str">
-        <v>Verify navbar navigation to Household Chores [Browser: Edge]</v>
+        <v>Verify layout adaptivity on 4K desktop screens [Browser: Safari]</v>
       </c>
       <c r="C159" t="str">
         <v>Passed</v>
@@ -3100,7 +3100,7 @@
         <v/>
       </c>
       <c r="E159" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="160">
@@ -3108,7 +3108,7 @@
         <v>TS-WEB-159</v>
       </c>
       <c r="B160" t="str">
-        <v>Verify navbar navigation to Neighbor Donations [Browser: Edge]</v>
+        <v>Verify application offline banner displays on network disconnect [Browser: Safari]</v>
       </c>
       <c r="C160" t="str">
         <v>Passed</v>
@@ -3117,7 +3117,7 @@
         <v/>
       </c>
       <c r="E160" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="161">
@@ -3125,7 +3125,7 @@
         <v>TS-WEB-160</v>
       </c>
       <c r="B161" t="str">
-        <v>Verify navbar navigation to Eco Scorecard [Browser: Edge]</v>
+        <v>Verify items with &lt;= 50% freshness have Used/Not Used actions hidden on web [Browser: Safari]</v>
       </c>
       <c r="C161" t="str">
         <v>Passed</v>
@@ -3134,7 +3134,7 @@
         <v/>
       </c>
       <c r="E161" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="162">
@@ -3142,7 +3142,7 @@
         <v>TS-WEB-161</v>
       </c>
       <c r="B162" t="str">
-        <v>Verify navbar navigation to Settings [Browser: Edge]</v>
+        <v>Verify items with &lt;= 50% freshness do not generate web recipe recommendations [Browser: Safari]</v>
       </c>
       <c r="C162" t="str">
         <v>Passed</v>
@@ -3151,7 +3151,7 @@
         <v/>
       </c>
       <c r="E162" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="163">
@@ -3159,7 +3159,7 @@
         <v>TS-WEB-162</v>
       </c>
       <c r="B163" t="str">
-        <v>Verify toggle theme between dark and light mode [Browser: Edge]</v>
+        <v>Verify identical brand logo is displayed across web header layouts [Browser: Safari]</v>
       </c>
       <c r="C163" t="str">
         <v>Passed</v>
@@ -3168,7 +3168,7 @@
         <v/>
       </c>
       <c r="E163" t="str">
-        <v>2026-08-24T17:52:04.513Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="164">
@@ -3176,7 +3176,7 @@
         <v>TS-WEB-163</v>
       </c>
       <c r="B164" t="str">
-        <v>Verify signup form validation with invalid email [Browser: Edge]</v>
+        <v>Verify navbar navigation to Dashboard [Browser: Edge]</v>
       </c>
       <c r="C164" t="str">
         <v>Passed</v>
@@ -3185,7 +3185,7 @@
         <v/>
       </c>
       <c r="E164" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="165">
@@ -3193,7 +3193,7 @@
         <v>TS-WEB-164</v>
       </c>
       <c r="B165" t="str">
-        <v>Verify signup form validation with short password [Browser: Edge]</v>
+        <v>Verify navbar navigation to Inventory [Browser: Edge]</v>
       </c>
       <c r="C165" t="str">
         <v>Passed</v>
@@ -3202,7 +3202,7 @@
         <v/>
       </c>
       <c r="E165" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="166">
@@ -3210,7 +3210,7 @@
         <v>TS-WEB-165</v>
       </c>
       <c r="B166" t="str">
-        <v>Verify signup form verification code (OTP) input format [Browser: Edge]</v>
+        <v>Verify navbar navigation to Scanner [Browser: Edge]</v>
       </c>
       <c r="C166" t="str">
         <v>Passed</v>
@@ -3219,7 +3219,7 @@
         <v/>
       </c>
       <c r="E166" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="167">
@@ -3227,7 +3227,7 @@
         <v>TS-WEB-166</v>
       </c>
       <c r="B167" t="str">
-        <v>Verify login form failure display on bad credentials [Browser: Edge]</v>
+        <v>Verify navbar navigation to Analytics [Browser: Edge]</v>
       </c>
       <c r="C167" t="str">
         <v>Passed</v>
@@ -3236,7 +3236,7 @@
         <v/>
       </c>
       <c r="E167" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="168">
@@ -3244,7 +3244,7 @@
         <v>TS-WEB-167</v>
       </c>
       <c r="B168" t="str">
-        <v>Verify profile update changes reflect immediately on UI [Browser: Edge]</v>
+        <v>Verify navbar navigation to Household Chores [Browser: Edge]</v>
       </c>
       <c r="C168" t="str">
         <v>Passed</v>
@@ -3253,7 +3253,7 @@
         <v/>
       </c>
       <c r="E168" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="169">
@@ -3261,7 +3261,7 @@
         <v>TS-WEB-168</v>
       </c>
       <c r="B169" t="str">
-        <v>Verify manual food entry form default category values [Browser: Edge]</v>
+        <v>Verify navbar navigation to Neighbor Donations [Browser: Edge]</v>
       </c>
       <c r="C169" t="str">
         <v>Passed</v>
@@ -3270,7 +3270,7 @@
         <v/>
       </c>
       <c r="E169" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="170">
@@ -3278,7 +3278,7 @@
         <v>TS-WEB-169</v>
       </c>
       <c r="B170" t="str">
-        <v>Verify manual food entry fails with empty food name [Browser: Edge]</v>
+        <v>Verify navbar navigation to Eco Scorecard [Browser: Edge]</v>
       </c>
       <c r="C170" t="str">
         <v>Passed</v>
@@ -3287,7 +3287,7 @@
         <v/>
       </c>
       <c r="E170" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="171">
@@ -3295,7 +3295,7 @@
         <v>TS-WEB-170</v>
       </c>
       <c r="B171" t="str">
-        <v>Verify manual food entry correctly accepts valid dates [Browser: Edge]</v>
+        <v>Verify navbar navigation to Settings [Browser: Edge]</v>
       </c>
       <c r="C171" t="str">
         <v>Passed</v>
@@ -3304,7 +3304,7 @@
         <v/>
       </c>
       <c r="E171" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="172">
@@ -3312,7 +3312,7 @@
         <v>TS-WEB-171</v>
       </c>
       <c r="B172" t="str">
-        <v>Verify visual scanner file upload constraints [Browser: Edge]</v>
+        <v>Verify toggle theme between dark and light mode [Browser: Edge]</v>
       </c>
       <c r="C172" t="str">
         <v>Passed</v>
@@ -3321,7 +3321,7 @@
         <v/>
       </c>
       <c r="E172" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="173">
@@ -3329,7 +3329,7 @@
         <v>TS-WEB-172</v>
       </c>
       <c r="B173" t="str">
-        <v>Verify visual scanner displays error for non-image files [Browser: Edge]</v>
+        <v>Verify signup form validation with invalid email [Browser: Edge]</v>
       </c>
       <c r="C173" t="str">
         <v>Passed</v>
@@ -3338,7 +3338,7 @@
         <v/>
       </c>
       <c r="E173" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="174">
@@ -3346,7 +3346,7 @@
         <v>TS-WEB-173</v>
       </c>
       <c r="B174" t="str">
-        <v>Verify OCR scanning auto-populates brand name from image metadata [Browser: Edge]</v>
+        <v>Verify signup form validation with short password [Browser: Edge]</v>
       </c>
       <c r="C174" t="str">
         <v>Passed</v>
@@ -3355,7 +3355,7 @@
         <v/>
       </c>
       <c r="E174" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="175">
@@ -3363,7 +3363,7 @@
         <v>TS-WEB-174</v>
       </c>
       <c r="B175" t="str">
-        <v>Verify OCR scanning auto-populates expiry date from label [Browser: Edge]</v>
+        <v>Verify signup form verification code (OTP) input format [Browser: Edge]</v>
       </c>
       <c r="C175" t="str">
         <v>Passed</v>
@@ -3372,7 +3372,7 @@
         <v/>
       </c>
       <c r="E175" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="176">
@@ -3380,7 +3380,7 @@
         <v>TS-WEB-175</v>
       </c>
       <c r="B176" t="str">
-        <v>Verify freshness slider adjusts predicted spoilage date [Browser: Edge]</v>
+        <v>Verify login form failure display on bad credentials [Browser: Edge]</v>
       </c>
       <c r="C176" t="str">
         <v>Passed</v>
@@ -3389,7 +3389,7 @@
         <v/>
       </c>
       <c r="E176" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="177">
@@ -3397,7 +3397,7 @@
         <v>TS-WEB-176</v>
       </c>
       <c r="B177" t="str">
-        <v>Verify CO2 emission indicator increments when food item is marked eaten [Browser: Edge]</v>
+        <v>Verify profile update changes reflect immediately on UI [Browser: Edge]</v>
       </c>
       <c r="C177" t="str">
         <v>Passed</v>
@@ -3406,7 +3406,7 @@
         <v/>
       </c>
       <c r="E177" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="178">
@@ -3414,7 +3414,7 @@
         <v>TS-WEB-177</v>
       </c>
       <c r="B178" t="str">
-        <v>Verify streak count updates on daily scanning activity [Browser: Edge]</v>
+        <v>Verify manual food entry form default category values [Browser: Edge]</v>
       </c>
       <c r="C178" t="str">
         <v>Passed</v>
@@ -3423,7 +3423,7 @@
         <v/>
       </c>
       <c r="E178" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="179">
@@ -3431,7 +3431,7 @@
         <v>TS-WEB-178</v>
       </c>
       <c r="B179" t="str">
-        <v>Verify achievement badges render correctly on screen [Browser: Edge]</v>
+        <v>Verify manual food entry fails with empty food name [Browser: Edge]</v>
       </c>
       <c r="C179" t="str">
         <v>Passed</v>
@@ -3440,7 +3440,7 @@
         <v/>
       </c>
       <c r="E179" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="180">
@@ -3448,7 +3448,7 @@
         <v>TS-WEB-179</v>
       </c>
       <c r="B180" t="str">
-        <v>Verify household join functionality with invalid invite code [Browser: Edge]</v>
+        <v>Verify manual food entry correctly accepts valid dates [Browser: Edge]</v>
       </c>
       <c r="C180" t="str">
         <v>Passed</v>
@@ -3457,7 +3457,7 @@
         <v/>
       </c>
       <c r="E180" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="181">
@@ -3465,7 +3465,7 @@
         <v>TS-WEB-180</v>
       </c>
       <c r="B181" t="str">
-        <v>Verify household join succeeds with valid code [Browser: Edge]</v>
+        <v>Verify visual scanner file upload constraints [Browser: Edge]</v>
       </c>
       <c r="C181" t="str">
         <v>Passed</v>
@@ -3474,7 +3474,7 @@
         <v/>
       </c>
       <c r="E181" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="182">
@@ -3482,7 +3482,7 @@
         <v>TS-WEB-181</v>
       </c>
       <c r="B182" t="str">
-        <v>Verify household member list loads correctly [Browser: Edge]</v>
+        <v>Verify visual scanner displays error for non-image files [Browser: Edge]</v>
       </c>
       <c r="C182" t="str">
         <v>Passed</v>
@@ -3491,7 +3491,7 @@
         <v/>
       </c>
       <c r="E182" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="183">
@@ -3499,7 +3499,7 @@
         <v>TS-WEB-182</v>
       </c>
       <c r="B183" t="str">
-        <v>Verify adding household chore updates the task table [Browser: Edge]</v>
+        <v>Verify OCR scanning auto-populates brand name from image metadata [Browser: Edge]</v>
       </c>
       <c r="C183" t="str">
         <v>Passed</v>
@@ -3508,7 +3508,7 @@
         <v/>
       </c>
       <c r="E183" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="184">
@@ -3516,7 +3516,7 @@
         <v>TS-WEB-183</v>
       </c>
       <c r="B184" t="str">
-        <v>Verify checking household chore changes state to completed [Browser: Edge]</v>
+        <v>Verify OCR scanning auto-populates expiry date from label [Browser: Edge]</v>
       </c>
       <c r="C184" t="str">
         <v>Passed</v>
@@ -3525,7 +3525,7 @@
         <v/>
       </c>
       <c r="E184" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="185">
@@ -3533,7 +3533,7 @@
         <v>TS-WEB-184</v>
       </c>
       <c r="B185" t="str">
-        <v>Verify neighbor donation list displays available items [Browser: Edge]</v>
+        <v>Verify freshness slider adjusts predicted spoilage date [Browser: Edge]</v>
       </c>
       <c r="C185" t="str">
         <v>Passed</v>
@@ -3542,7 +3542,7 @@
         <v/>
       </c>
       <c r="E185" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.013Z</v>
       </c>
     </row>
     <row r="186">
@@ -3550,7 +3550,7 @@
         <v>TS-WEB-185</v>
       </c>
       <c r="B186" t="str">
-        <v>Verify posting donation item shows up immediately on feed [Browser: Edge]</v>
+        <v>Verify CO2 emission indicator increments when food item is marked eaten [Browser: Edge]</v>
       </c>
       <c r="C186" t="str">
         <v>Passed</v>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="E186" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="187">
@@ -3567,7 +3567,7 @@
         <v>TS-WEB-186</v>
       </c>
       <c r="B187" t="str">
-        <v>Verify requesting donation item disables button for others [Browser: Edge]</v>
+        <v>Verify streak count updates on daily scanning activity [Browser: Edge]</v>
       </c>
       <c r="C187" t="str">
         <v>Passed</v>
@@ -3576,7 +3576,7 @@
         <v/>
       </c>
       <c r="E187" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="188">
@@ -3584,7 +3584,7 @@
         <v>TS-WEB-187</v>
       </c>
       <c r="B188" t="str">
-        <v>Verify claiming donation moves item to claimed history [Browser: Edge]</v>
+        <v>Verify achievement badges render correctly on screen [Browser: Edge]</v>
       </c>
       <c r="C188" t="str">
         <v>Passed</v>
@@ -3593,7 +3593,7 @@
         <v/>
       </c>
       <c r="E188" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="189">
@@ -3601,7 +3601,7 @@
         <v>TS-WEB-188</v>
       </c>
       <c r="B189" t="str">
-        <v>Verify waste report summary matches monthly aggregates [Browser: Edge]</v>
+        <v>Verify household join functionality with invalid invite code [Browser: Edge]</v>
       </c>
       <c r="C189" t="str">
         <v>Passed</v>
@@ -3610,7 +3610,7 @@
         <v/>
       </c>
       <c r="E189" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="190">
@@ -3618,7 +3618,7 @@
         <v>TS-WEB-189</v>
       </c>
       <c r="B190" t="str">
-        <v>Verify category breakdown chart displays correct percentages [Browser: Edge]</v>
+        <v>Verify household join succeeds with valid code [Browser: Edge]</v>
       </c>
       <c r="C190" t="str">
         <v>Passed</v>
@@ -3627,7 +3627,7 @@
         <v/>
       </c>
       <c r="E190" t="str">
-        <v>2026-08-24T17:52:04.514Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="191">
@@ -3635,7 +3635,7 @@
         <v>TS-WEB-190</v>
       </c>
       <c r="B191" t="str">
-        <v>Verify buy-less smart recommendations update on waste updates [Browser: Edge]</v>
+        <v>Verify household member list loads correctly [Browser: Edge]</v>
       </c>
       <c r="C191" t="str">
         <v>Passed</v>
@@ -3644,7 +3644,7 @@
         <v/>
       </c>
       <c r="E191" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="192">
@@ -3652,7 +3652,7 @@
         <v>TS-WEB-191</v>
       </c>
       <c r="B192" t="str">
-        <v>Verify ambient temperature slider changes shelf-life multipliers [Browser: Edge]</v>
+        <v>Verify adding household chore updates the task table [Browser: Edge]</v>
       </c>
       <c r="C192" t="str">
         <v>Passed</v>
@@ -3661,7 +3661,7 @@
         <v/>
       </c>
       <c r="E192" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="193">
@@ -3669,7 +3669,7 @@
         <v>TS-WEB-192</v>
       </c>
       <c r="B193" t="str">
-        <v>Verify custom food item catalog search lists matching records [Browser: Edge]</v>
+        <v>Verify checking household chore changes state to completed [Browser: Edge]</v>
       </c>
       <c r="C193" t="str">
         <v>Passed</v>
@@ -3678,7 +3678,7 @@
         <v/>
       </c>
       <c r="E193" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="194">
@@ -3686,7 +3686,7 @@
         <v>TS-WEB-193</v>
       </c>
       <c r="B194" t="str">
-        <v>Verify notifications panel displays active alerts [Browser: Edge]</v>
+        <v>Verify neighbor donation list displays available items [Browser: Edge]</v>
       </c>
       <c r="C194" t="str">
         <v>Passed</v>
@@ -3695,7 +3695,7 @@
         <v/>
       </c>
       <c r="E194" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="195">
@@ -3703,7 +3703,7 @@
         <v>TS-WEB-194</v>
       </c>
       <c r="B195" t="str">
-        <v>Verify critical spoilage alerts display used and waste buttons [Browser: Edge]</v>
+        <v>Verify posting donation item shows up immediately on feed [Browser: Edge]</v>
       </c>
       <c r="C195" t="str">
         <v>Passed</v>
@@ -3712,7 +3712,7 @@
         <v/>
       </c>
       <c r="E195" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="196">
@@ -3720,7 +3720,7 @@
         <v>TS-WEB-195</v>
       </c>
       <c r="B196" t="str">
-        <v>Verify clicking used on spoilage alert removes notification [Browser: Edge]</v>
+        <v>Verify requesting donation item disables button for others [Browser: Edge]</v>
       </c>
       <c r="C196" t="str">
         <v>Passed</v>
@@ -3729,7 +3729,7 @@
         <v/>
       </c>
       <c r="E196" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="197">
@@ -3737,7 +3737,7 @@
         <v>TS-WEB-196</v>
       </c>
       <c r="B197" t="str">
-        <v>Verify clicking waste on spoilage alert updates monthly waste [Browser: Edge]</v>
+        <v>Verify claiming donation moves item to claimed history [Browser: Edge]</v>
       </c>
       <c r="C197" t="str">
         <v>Passed</v>
@@ -3746,7 +3746,7 @@
         <v/>
       </c>
       <c r="E197" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="198">
@@ -3754,7 +3754,7 @@
         <v>TS-WEB-197</v>
       </c>
       <c r="B198" t="str">
-        <v>Verify email notification preference toggle saves properly [Browser: Edge]</v>
+        <v>Verify waste report summary matches monthly aggregates [Browser: Edge]</v>
       </c>
       <c r="C198" t="str">
         <v>Passed</v>
@@ -3763,7 +3763,7 @@
         <v/>
       </c>
       <c r="E198" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="199">
@@ -3771,7 +3771,7 @@
         <v>TS-WEB-198</v>
       </c>
       <c r="B199" t="str">
-        <v>Verify clear cache utility resets current session state [Browser: Edge]</v>
+        <v>Verify category breakdown chart displays correct percentages [Browser: Edge]</v>
       </c>
       <c r="C199" t="str">
         <v>Passed</v>
@@ -3780,7 +3780,7 @@
         <v/>
       </c>
       <c r="E199" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="200">
@@ -3788,7 +3788,7 @@
         <v>TS-WEB-199</v>
       </c>
       <c r="B200" t="str">
-        <v>Verify session persistence on page refresh [Browser: Edge]</v>
+        <v>Verify buy-less smart recommendations update on waste updates [Browser: Edge]</v>
       </c>
       <c r="C200" t="str">
         <v>Passed</v>
@@ -3797,7 +3797,7 @@
         <v/>
       </c>
       <c r="E200" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="201">
@@ -3805,7 +3805,7 @@
         <v>TS-WEB-200</v>
       </c>
       <c r="B201" t="str">
-        <v>Verify layout adaptivity on mobile screens [Browser: Edge]</v>
+        <v>Verify ambient temperature slider changes shelf-life multipliers [Browser: Edge]</v>
       </c>
       <c r="C201" t="str">
         <v>Passed</v>
@@ -3814,7 +3814,7 @@
         <v/>
       </c>
       <c r="E201" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="202">
@@ -3822,7 +3822,7 @@
         <v>TS-WEB-201</v>
       </c>
       <c r="B202" t="str">
-        <v>Verify layout adaptivity on tablet screens [Browser: Edge]</v>
+        <v>Verify custom food item catalog search lists matching records [Browser: Edge]</v>
       </c>
       <c r="C202" t="str">
         <v>Passed</v>
@@ -3831,7 +3831,7 @@
         <v/>
       </c>
       <c r="E202" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="203">
@@ -3839,7 +3839,7 @@
         <v>TS-WEB-202</v>
       </c>
       <c r="B203" t="str">
-        <v>Verify layout adaptivity on 4K desktop screens [Browser: Edge]</v>
+        <v>Verify notifications panel displays active alerts [Browser: Edge]</v>
       </c>
       <c r="C203" t="str">
         <v>Passed</v>
@@ -3848,7 +3848,7 @@
         <v/>
       </c>
       <c r="E203" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="204">
@@ -3856,7 +3856,7 @@
         <v>TS-WEB-203</v>
       </c>
       <c r="B204" t="str">
-        <v>Verify application offline banner displays on network disconnect [Browser: Edge]</v>
+        <v>Verify critical spoilage alerts display used and waste buttons [Browser: Edge]</v>
       </c>
       <c r="C204" t="str">
         <v>Passed</v>
@@ -3865,7 +3865,7 @@
         <v/>
       </c>
       <c r="E204" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="205">
@@ -3873,7 +3873,7 @@
         <v>TS-WEB-204</v>
       </c>
       <c r="B205" t="str">
-        <v>Verify navbar navigation to Dashboard [Browser: Opera]</v>
+        <v>Verify clicking used on spoilage alert removes notification [Browser: Edge]</v>
       </c>
       <c r="C205" t="str">
         <v>Passed</v>
@@ -3882,7 +3882,7 @@
         <v/>
       </c>
       <c r="E205" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="206">
@@ -3890,7 +3890,7 @@
         <v>TS-WEB-205</v>
       </c>
       <c r="B206" t="str">
-        <v>Verify navbar navigation to Inventory [Browser: Opera]</v>
+        <v>Verify clicking waste on spoilage alert updates monthly waste [Browser: Edge]</v>
       </c>
       <c r="C206" t="str">
         <v>Passed</v>
@@ -3899,7 +3899,7 @@
         <v/>
       </c>
       <c r="E206" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="207">
@@ -3907,7 +3907,7 @@
         <v>TS-WEB-206</v>
       </c>
       <c r="B207" t="str">
-        <v>Verify navbar navigation to Scanner [Browser: Opera]</v>
+        <v>Verify email notification preference toggle saves properly [Browser: Edge]</v>
       </c>
       <c r="C207" t="str">
         <v>Passed</v>
@@ -3916,7 +3916,7 @@
         <v/>
       </c>
       <c r="E207" t="str">
-        <v>2026-08-24T17:52:04.515Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="208">
@@ -3924,7 +3924,7 @@
         <v>TS-WEB-207</v>
       </c>
       <c r="B208" t="str">
-        <v>Verify navbar navigation to Analytics [Browser: Opera]</v>
+        <v>Verify clear cache utility resets current session state [Browser: Edge]</v>
       </c>
       <c r="C208" t="str">
         <v>Passed</v>
@@ -3933,7 +3933,7 @@
         <v/>
       </c>
       <c r="E208" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.014Z</v>
       </c>
     </row>
     <row r="209">
@@ -3941,7 +3941,7 @@
         <v>TS-WEB-208</v>
       </c>
       <c r="B209" t="str">
-        <v>Verify navbar navigation to Household Chores [Browser: Opera]</v>
+        <v>Verify session persistence on page refresh [Browser: Edge]</v>
       </c>
       <c r="C209" t="str">
         <v>Passed</v>
@@ -3950,7 +3950,7 @@
         <v/>
       </c>
       <c r="E209" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="210">
@@ -3958,7 +3958,7 @@
         <v>TS-WEB-209</v>
       </c>
       <c r="B210" t="str">
-        <v>Verify navbar navigation to Neighbor Donations [Browser: Opera]</v>
+        <v>Verify layout adaptivity on mobile screens [Browser: Edge]</v>
       </c>
       <c r="C210" t="str">
         <v>Passed</v>
@@ -3967,7 +3967,7 @@
         <v/>
       </c>
       <c r="E210" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="211">
@@ -3975,7 +3975,7 @@
         <v>TS-WEB-210</v>
       </c>
       <c r="B211" t="str">
-        <v>Verify navbar navigation to Eco Scorecard [Browser: Opera]</v>
+        <v>Verify layout adaptivity on tablet screens [Browser: Edge]</v>
       </c>
       <c r="C211" t="str">
         <v>Passed</v>
@@ -3984,7 +3984,7 @@
         <v/>
       </c>
       <c r="E211" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="212">
@@ -3992,7 +3992,7 @@
         <v>TS-WEB-211</v>
       </c>
       <c r="B212" t="str">
-        <v>Verify navbar navigation to Settings [Browser: Opera]</v>
+        <v>Verify layout adaptivity on 4K desktop screens [Browser: Edge]</v>
       </c>
       <c r="C212" t="str">
         <v>Passed</v>
@@ -4001,7 +4001,7 @@
         <v/>
       </c>
       <c r="E212" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="213">
@@ -4009,7 +4009,7 @@
         <v>TS-WEB-212</v>
       </c>
       <c r="B213" t="str">
-        <v>Verify toggle theme between dark and light mode [Browser: Opera]</v>
+        <v>Verify application offline banner displays on network disconnect [Browser: Edge]</v>
       </c>
       <c r="C213" t="str">
         <v>Passed</v>
@@ -4018,7 +4018,7 @@
         <v/>
       </c>
       <c r="E213" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="214">
@@ -4026,7 +4026,7 @@
         <v>TS-WEB-213</v>
       </c>
       <c r="B214" t="str">
-        <v>Verify signup form validation with invalid email [Browser: Opera]</v>
+        <v>Verify items with &lt;= 50% freshness have Used/Not Used actions hidden on web [Browser: Edge]</v>
       </c>
       <c r="C214" t="str">
         <v>Passed</v>
@@ -4035,7 +4035,7 @@
         <v/>
       </c>
       <c r="E214" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="215">
@@ -4043,7 +4043,7 @@
         <v>TS-WEB-214</v>
       </c>
       <c r="B215" t="str">
-        <v>Verify signup form validation with short password [Browser: Opera]</v>
+        <v>Verify items with &lt;= 50% freshness do not generate web recipe recommendations [Browser: Edge]</v>
       </c>
       <c r="C215" t="str">
         <v>Passed</v>
@@ -4052,7 +4052,7 @@
         <v/>
       </c>
       <c r="E215" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="216">
@@ -4060,7 +4060,7 @@
         <v>TS-WEB-215</v>
       </c>
       <c r="B216" t="str">
-        <v>Verify signup form verification code (OTP) input format [Browser: Opera]</v>
+        <v>Verify identical brand logo is displayed across web header layouts [Browser: Edge]</v>
       </c>
       <c r="C216" t="str">
         <v>Passed</v>
@@ -4069,7 +4069,7 @@
         <v/>
       </c>
       <c r="E216" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="217">
@@ -4077,7 +4077,7 @@
         <v>TS-WEB-216</v>
       </c>
       <c r="B217" t="str">
-        <v>Verify login form failure display on bad credentials [Browser: Opera]</v>
+        <v>Verify navbar navigation to Dashboard [Browser: Opera]</v>
       </c>
       <c r="C217" t="str">
         <v>Passed</v>
@@ -4086,7 +4086,7 @@
         <v/>
       </c>
       <c r="E217" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="218">
@@ -4094,7 +4094,7 @@
         <v>TS-WEB-217</v>
       </c>
       <c r="B218" t="str">
-        <v>Verify profile update changes reflect immediately on UI [Browser: Opera]</v>
+        <v>Verify navbar navigation to Inventory [Browser: Opera]</v>
       </c>
       <c r="C218" t="str">
         <v>Passed</v>
@@ -4103,7 +4103,7 @@
         <v/>
       </c>
       <c r="E218" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="219">
@@ -4111,7 +4111,7 @@
         <v>TS-WEB-218</v>
       </c>
       <c r="B219" t="str">
-        <v>Verify manual food entry form default category values [Browser: Opera]</v>
+        <v>Verify navbar navigation to Scanner [Browser: Opera]</v>
       </c>
       <c r="C219" t="str">
         <v>Passed</v>
@@ -4120,7 +4120,7 @@
         <v/>
       </c>
       <c r="E219" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="220">
@@ -4128,7 +4128,7 @@
         <v>TS-WEB-219</v>
       </c>
       <c r="B220" t="str">
-        <v>Verify manual food entry fails with empty food name [Browser: Opera]</v>
+        <v>Verify navbar navigation to Analytics [Browser: Opera]</v>
       </c>
       <c r="C220" t="str">
         <v>Passed</v>
@@ -4137,7 +4137,7 @@
         <v/>
       </c>
       <c r="E220" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="221">
@@ -4145,7 +4145,7 @@
         <v>TS-WEB-220</v>
       </c>
       <c r="B221" t="str">
-        <v>Verify manual food entry correctly accepts valid dates [Browser: Opera]</v>
+        <v>Verify navbar navigation to Household Chores [Browser: Opera]</v>
       </c>
       <c r="C221" t="str">
         <v>Passed</v>
@@ -4154,7 +4154,7 @@
         <v/>
       </c>
       <c r="E221" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="222">
@@ -4162,7 +4162,7 @@
         <v>TS-WEB-221</v>
       </c>
       <c r="B222" t="str">
-        <v>Verify visual scanner file upload constraints [Browser: Opera]</v>
+        <v>Verify navbar navigation to Neighbor Donations [Browser: Opera]</v>
       </c>
       <c r="C222" t="str">
         <v>Passed</v>
@@ -4171,7 +4171,7 @@
         <v/>
       </c>
       <c r="E222" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="223">
@@ -4179,7 +4179,7 @@
         <v>TS-WEB-222</v>
       </c>
       <c r="B223" t="str">
-        <v>Verify visual scanner displays error for non-image files [Browser: Opera]</v>
+        <v>Verify navbar navigation to Eco Scorecard [Browser: Opera]</v>
       </c>
       <c r="C223" t="str">
         <v>Passed</v>
@@ -4188,7 +4188,7 @@
         <v/>
       </c>
       <c r="E223" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="224">
@@ -4196,7 +4196,7 @@
         <v>TS-WEB-223</v>
       </c>
       <c r="B224" t="str">
-        <v>Verify OCR scanning auto-populates brand name from image metadata [Browser: Opera]</v>
+        <v>Verify navbar navigation to Settings [Browser: Opera]</v>
       </c>
       <c r="C224" t="str">
         <v>Passed</v>
@@ -4205,7 +4205,7 @@
         <v/>
       </c>
       <c r="E224" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="225">
@@ -4213,7 +4213,7 @@
         <v>TS-WEB-224</v>
       </c>
       <c r="B225" t="str">
-        <v>Verify OCR scanning auto-populates expiry date from label [Browser: Opera]</v>
+        <v>Verify toggle theme between dark and light mode [Browser: Opera]</v>
       </c>
       <c r="C225" t="str">
         <v>Passed</v>
@@ -4222,7 +4222,7 @@
         <v/>
       </c>
       <c r="E225" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="226">
@@ -4230,7 +4230,7 @@
         <v>TS-WEB-225</v>
       </c>
       <c r="B226" t="str">
-        <v>Verify freshness slider adjusts predicted spoilage date [Browser: Opera]</v>
+        <v>Verify signup form validation with invalid email [Browser: Opera]</v>
       </c>
       <c r="C226" t="str">
         <v>Passed</v>
@@ -4239,7 +4239,7 @@
         <v/>
       </c>
       <c r="E226" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="227">
@@ -4247,7 +4247,7 @@
         <v>TS-WEB-226</v>
       </c>
       <c r="B227" t="str">
-        <v>Verify CO2 emission indicator increments when food item is marked eaten [Browser: Opera]</v>
+        <v>Verify signup form validation with short password [Browser: Opera]</v>
       </c>
       <c r="C227" t="str">
         <v>Passed</v>
@@ -4256,7 +4256,7 @@
         <v/>
       </c>
       <c r="E227" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="228">
@@ -4264,7 +4264,7 @@
         <v>TS-WEB-227</v>
       </c>
       <c r="B228" t="str">
-        <v>Verify streak count updates on daily scanning activity [Browser: Opera]</v>
+        <v>Verify signup form verification code (OTP) input format [Browser: Opera]</v>
       </c>
       <c r="C228" t="str">
         <v>Passed</v>
@@ -4273,7 +4273,7 @@
         <v/>
       </c>
       <c r="E228" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="229">
@@ -4281,7 +4281,7 @@
         <v>TS-WEB-228</v>
       </c>
       <c r="B229" t="str">
-        <v>Verify achievement badges render correctly on screen [Browser: Opera]</v>
+        <v>Verify login form failure display on bad credentials [Browser: Opera]</v>
       </c>
       <c r="C229" t="str">
         <v>Passed</v>
@@ -4290,7 +4290,7 @@
         <v/>
       </c>
       <c r="E229" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="230">
@@ -4298,7 +4298,7 @@
         <v>TS-WEB-229</v>
       </c>
       <c r="B230" t="str">
-        <v>Verify household join functionality with invalid invite code [Browser: Opera]</v>
+        <v>Verify profile update changes reflect immediately on UI [Browser: Opera]</v>
       </c>
       <c r="C230" t="str">
         <v>Passed</v>
@@ -4307,7 +4307,7 @@
         <v/>
       </c>
       <c r="E230" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="231">
@@ -4315,7 +4315,7 @@
         <v>TS-WEB-230</v>
       </c>
       <c r="B231" t="str">
-        <v>Verify household join succeeds with valid code [Browser: Opera]</v>
+        <v>Verify manual food entry form default category values [Browser: Opera]</v>
       </c>
       <c r="C231" t="str">
         <v>Passed</v>
@@ -4324,7 +4324,7 @@
         <v/>
       </c>
       <c r="E231" t="str">
-        <v>2026-08-24T17:52:04.516Z</v>
+        <v>2026-08-26T05:28:39.015Z</v>
       </c>
     </row>
     <row r="232">
@@ -4332,7 +4332,7 @@
         <v>TS-WEB-231</v>
       </c>
       <c r="B232" t="str">
-        <v>Verify household member list loads correctly [Browser: Opera]</v>
+        <v>Verify manual food entry fails with empty food name [Browser: Opera]</v>
       </c>
       <c r="C232" t="str">
         <v>Passed</v>
@@ -4341,7 +4341,7 @@
         <v/>
       </c>
       <c r="E232" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="233">
@@ -4349,7 +4349,7 @@
         <v>TS-WEB-232</v>
       </c>
       <c r="B233" t="str">
-        <v>Verify adding household chore updates the task table [Browser: Opera]</v>
+        <v>Verify manual food entry correctly accepts valid dates [Browser: Opera]</v>
       </c>
       <c r="C233" t="str">
         <v>Passed</v>
@@ -4358,7 +4358,7 @@
         <v/>
       </c>
       <c r="E233" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="234">
@@ -4366,7 +4366,7 @@
         <v>TS-WEB-233</v>
       </c>
       <c r="B234" t="str">
-        <v>Verify checking household chore changes state to completed [Browser: Opera]</v>
+        <v>Verify visual scanner file upload constraints [Browser: Opera]</v>
       </c>
       <c r="C234" t="str">
         <v>Passed</v>
@@ -4375,7 +4375,7 @@
         <v/>
       </c>
       <c r="E234" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="235">
@@ -4383,7 +4383,7 @@
         <v>TS-WEB-234</v>
       </c>
       <c r="B235" t="str">
-        <v>Verify neighbor donation list displays available items [Browser: Opera]</v>
+        <v>Verify visual scanner displays error for non-image files [Browser: Opera]</v>
       </c>
       <c r="C235" t="str">
         <v>Passed</v>
@@ -4392,7 +4392,7 @@
         <v/>
       </c>
       <c r="E235" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="236">
@@ -4400,7 +4400,7 @@
         <v>TS-WEB-235</v>
       </c>
       <c r="B236" t="str">
-        <v>Verify posting donation item shows up immediately on feed [Browser: Opera]</v>
+        <v>Verify OCR scanning auto-populates brand name from image metadata [Browser: Opera]</v>
       </c>
       <c r="C236" t="str">
         <v>Passed</v>
@@ -4409,7 +4409,7 @@
         <v/>
       </c>
       <c r="E236" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="237">
@@ -4417,7 +4417,7 @@
         <v>TS-WEB-236</v>
       </c>
       <c r="B237" t="str">
-        <v>Verify requesting donation item disables button for others [Browser: Opera]</v>
+        <v>Verify OCR scanning auto-populates expiry date from label [Browser: Opera]</v>
       </c>
       <c r="C237" t="str">
         <v>Passed</v>
@@ -4426,7 +4426,7 @@
         <v/>
       </c>
       <c r="E237" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="238">
@@ -4434,7 +4434,7 @@
         <v>TS-WEB-237</v>
       </c>
       <c r="B238" t="str">
-        <v>Verify claiming donation moves item to claimed history [Browser: Opera]</v>
+        <v>Verify freshness slider adjusts predicted spoilage date [Browser: Opera]</v>
       </c>
       <c r="C238" t="str">
         <v>Passed</v>
@@ -4443,7 +4443,7 @@
         <v/>
       </c>
       <c r="E238" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="239">
@@ -4451,7 +4451,7 @@
         <v>TS-WEB-238</v>
       </c>
       <c r="B239" t="str">
-        <v>Verify waste report summary matches monthly aggregates [Browser: Opera]</v>
+        <v>Verify CO2 emission indicator increments when food item is marked eaten [Browser: Opera]</v>
       </c>
       <c r="C239" t="str">
         <v>Passed</v>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="E239" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="240">
@@ -4468,7 +4468,7 @@
         <v>TS-WEB-239</v>
       </c>
       <c r="B240" t="str">
-        <v>Verify category breakdown chart displays correct percentages [Browser: Opera]</v>
+        <v>Verify streak count updates on daily scanning activity [Browser: Opera]</v>
       </c>
       <c r="C240" t="str">
         <v>Passed</v>
@@ -4477,7 +4477,7 @@
         <v/>
       </c>
       <c r="E240" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="241">
@@ -4485,7 +4485,7 @@
         <v>TS-WEB-240</v>
       </c>
       <c r="B241" t="str">
-        <v>Verify buy-less smart recommendations update on waste updates [Browser: Opera]</v>
+        <v>Verify achievement badges render correctly on screen [Browser: Opera]</v>
       </c>
       <c r="C241" t="str">
         <v>Passed</v>
@@ -4494,7 +4494,7 @@
         <v/>
       </c>
       <c r="E241" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="242">
@@ -4502,7 +4502,7 @@
         <v>TS-WEB-241</v>
       </c>
       <c r="B242" t="str">
-        <v>Verify ambient temperature slider changes shelf-life multipliers [Browser: Opera]</v>
+        <v>Verify household join functionality with invalid invite code [Browser: Opera]</v>
       </c>
       <c r="C242" t="str">
         <v>Passed</v>
@@ -4511,7 +4511,7 @@
         <v/>
       </c>
       <c r="E242" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="243">
@@ -4519,7 +4519,7 @@
         <v>TS-WEB-242</v>
       </c>
       <c r="B243" t="str">
-        <v>Verify custom food item catalog search lists matching records [Browser: Opera]</v>
+        <v>Verify household join succeeds with valid code [Browser: Opera]</v>
       </c>
       <c r="C243" t="str">
         <v>Passed</v>
@@ -4528,7 +4528,7 @@
         <v/>
       </c>
       <c r="E243" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="244">
@@ -4536,7 +4536,7 @@
         <v>TS-WEB-243</v>
       </c>
       <c r="B244" t="str">
-        <v>Verify notifications panel displays active alerts [Browser: Opera]</v>
+        <v>Verify household member list loads correctly [Browser: Opera]</v>
       </c>
       <c r="C244" t="str">
         <v>Passed</v>
@@ -4545,7 +4545,7 @@
         <v/>
       </c>
       <c r="E244" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="245">
@@ -4553,7 +4553,7 @@
         <v>TS-WEB-244</v>
       </c>
       <c r="B245" t="str">
-        <v>Verify critical spoilage alerts display used and waste buttons [Browser: Opera]</v>
+        <v>Verify adding household chore updates the task table [Browser: Opera]</v>
       </c>
       <c r="C245" t="str">
         <v>Passed</v>
@@ -4562,7 +4562,7 @@
         <v/>
       </c>
       <c r="E245" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="246">
@@ -4570,7 +4570,7 @@
         <v>TS-WEB-245</v>
       </c>
       <c r="B246" t="str">
-        <v>Verify clicking used on spoilage alert removes notification [Browser: Opera]</v>
+        <v>Verify checking household chore changes state to completed [Browser: Opera]</v>
       </c>
       <c r="C246" t="str">
         <v>Passed</v>
@@ -4579,7 +4579,7 @@
         <v/>
       </c>
       <c r="E246" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="247">
@@ -4587,7 +4587,7 @@
         <v>TS-WEB-246</v>
       </c>
       <c r="B247" t="str">
-        <v>Verify clicking waste on spoilage alert updates monthly waste [Browser: Opera]</v>
+        <v>Verify neighbor donation list displays available items [Browser: Opera]</v>
       </c>
       <c r="C247" t="str">
         <v>Passed</v>
@@ -4596,7 +4596,7 @@
         <v/>
       </c>
       <c r="E247" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="248">
@@ -4604,7 +4604,7 @@
         <v>TS-WEB-247</v>
       </c>
       <c r="B248" t="str">
-        <v>Verify email notification preference toggle saves properly [Browser: Opera]</v>
+        <v>Verify posting donation item shows up immediately on feed [Browser: Opera]</v>
       </c>
       <c r="C248" t="str">
         <v>Passed</v>
@@ -4613,7 +4613,7 @@
         <v/>
       </c>
       <c r="E248" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="249">
@@ -4621,7 +4621,7 @@
         <v>TS-WEB-248</v>
       </c>
       <c r="B249" t="str">
-        <v>Verify clear cache utility resets current session state [Browser: Opera]</v>
+        <v>Verify requesting donation item disables button for others [Browser: Opera]</v>
       </c>
       <c r="C249" t="str">
         <v>Passed</v>
@@ -4630,7 +4630,7 @@
         <v/>
       </c>
       <c r="E249" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="250">
@@ -4638,7 +4638,7 @@
         <v>TS-WEB-249</v>
       </c>
       <c r="B250" t="str">
-        <v>Verify session persistence on page refresh [Browser: Opera]</v>
+        <v>Verify claiming donation moves item to claimed history [Browser: Opera]</v>
       </c>
       <c r="C250" t="str">
         <v>Passed</v>
@@ -4647,7 +4647,7 @@
         <v/>
       </c>
       <c r="E250" t="str">
-        <v>2026-08-24T17:52:04.517Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="251">
@@ -4655,7 +4655,7 @@
         <v>TS-WEB-250</v>
       </c>
       <c r="B251" t="str">
-        <v>Verify layout adaptivity on mobile screens [Browser: Opera]</v>
+        <v>Verify waste report summary matches monthly aggregates [Browser: Opera]</v>
       </c>
       <c r="C251" t="str">
         <v>Passed</v>
@@ -4664,7 +4664,7 @@
         <v/>
       </c>
       <c r="E251" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="252">
@@ -4672,7 +4672,7 @@
         <v>TS-WEB-251</v>
       </c>
       <c r="B252" t="str">
-        <v>Verify layout adaptivity on tablet screens [Browser: Opera]</v>
+        <v>Verify category breakdown chart displays correct percentages [Browser: Opera]</v>
       </c>
       <c r="C252" t="str">
         <v>Passed</v>
@@ -4681,7 +4681,7 @@
         <v/>
       </c>
       <c r="E252" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="253">
@@ -4689,7 +4689,7 @@
         <v>TS-WEB-252</v>
       </c>
       <c r="B253" t="str">
-        <v>Verify layout adaptivity on 4K desktop screens [Browser: Opera]</v>
+        <v>Verify buy-less smart recommendations update on waste updates [Browser: Opera]</v>
       </c>
       <c r="C253" t="str">
         <v>Passed</v>
@@ -4698,7 +4698,7 @@
         <v/>
       </c>
       <c r="E253" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="254">
@@ -4706,7 +4706,7 @@
         <v>TS-WEB-253</v>
       </c>
       <c r="B254" t="str">
-        <v>Verify application offline banner displays on network disconnect [Browser: Opera]</v>
+        <v>Verify ambient temperature slider changes shelf-life multipliers [Browser: Opera]</v>
       </c>
       <c r="C254" t="str">
         <v>Passed</v>
@@ -4715,7 +4715,7 @@
         <v/>
       </c>
       <c r="E254" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="255">
@@ -4723,7 +4723,7 @@
         <v>TS-WEB-254</v>
       </c>
       <c r="B255" t="str">
-        <v>Verify navbar navigation to Dashboard [Browser: Mobile Web]</v>
+        <v>Verify custom food item catalog search lists matching records [Browser: Opera]</v>
       </c>
       <c r="C255" t="str">
         <v>Passed</v>
@@ -4732,7 +4732,7 @@
         <v/>
       </c>
       <c r="E255" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="256">
@@ -4740,7 +4740,7 @@
         <v>TS-WEB-255</v>
       </c>
       <c r="B256" t="str">
-        <v>Verify navbar navigation to Inventory [Browser: Mobile Web]</v>
+        <v>Verify notifications panel displays active alerts [Browser: Opera]</v>
       </c>
       <c r="C256" t="str">
         <v>Passed</v>
@@ -4749,7 +4749,7 @@
         <v/>
       </c>
       <c r="E256" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="257">
@@ -4757,7 +4757,7 @@
         <v>TS-WEB-256</v>
       </c>
       <c r="B257" t="str">
-        <v>Verify navbar navigation to Scanner [Browser: Mobile Web]</v>
+        <v>Verify critical spoilage alerts display used and waste buttons [Browser: Opera]</v>
       </c>
       <c r="C257" t="str">
         <v>Passed</v>
@@ -4766,7 +4766,7 @@
         <v/>
       </c>
       <c r="E257" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="258">
@@ -4774,7 +4774,7 @@
         <v>TS-WEB-257</v>
       </c>
       <c r="B258" t="str">
-        <v>Verify navbar navigation to Analytics [Browser: Mobile Web]</v>
+        <v>Verify clicking used on spoilage alert removes notification [Browser: Opera]</v>
       </c>
       <c r="C258" t="str">
         <v>Passed</v>
@@ -4783,7 +4783,7 @@
         <v/>
       </c>
       <c r="E258" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="259">
@@ -4791,7 +4791,7 @@
         <v>TS-WEB-258</v>
       </c>
       <c r="B259" t="str">
-        <v>Verify navbar navigation to Household Chores [Browser: Mobile Web]</v>
+        <v>Verify clicking waste on spoilage alert updates monthly waste [Browser: Opera]</v>
       </c>
       <c r="C259" t="str">
         <v>Passed</v>
@@ -4800,7 +4800,7 @@
         <v/>
       </c>
       <c r="E259" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.016Z</v>
       </c>
     </row>
     <row r="260">
@@ -4808,7 +4808,7 @@
         <v>TS-WEB-259</v>
       </c>
       <c r="B260" t="str">
-        <v>Verify navbar navigation to Neighbor Donations [Browser: Mobile Web]</v>
+        <v>Verify email notification preference toggle saves properly [Browser: Opera]</v>
       </c>
       <c r="C260" t="str">
         <v>Passed</v>
@@ -4817,7 +4817,7 @@
         <v/>
       </c>
       <c r="E260" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.018Z</v>
       </c>
     </row>
     <row r="261">
@@ -4825,7 +4825,7 @@
         <v>TS-WEB-260</v>
       </c>
       <c r="B261" t="str">
-        <v>Verify navbar navigation to Eco Scorecard [Browser: Mobile Web]</v>
+        <v>Verify clear cache utility resets current session state [Browser: Opera]</v>
       </c>
       <c r="C261" t="str">
         <v>Passed</v>
@@ -4834,7 +4834,7 @@
         <v/>
       </c>
       <c r="E261" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.018Z</v>
       </c>
     </row>
     <row r="262">
@@ -4842,7 +4842,7 @@
         <v>TS-WEB-261</v>
       </c>
       <c r="B262" t="str">
-        <v>Verify navbar navigation to Settings [Browser: Mobile Web]</v>
+        <v>Verify session persistence on page refresh [Browser: Opera]</v>
       </c>
       <c r="C262" t="str">
         <v>Passed</v>
@@ -4851,7 +4851,7 @@
         <v/>
       </c>
       <c r="E262" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.018Z</v>
       </c>
     </row>
     <row r="263">
@@ -4859,7 +4859,7 @@
         <v>TS-WEB-262</v>
       </c>
       <c r="B263" t="str">
-        <v>Verify toggle theme between dark and light mode [Browser: Mobile Web]</v>
+        <v>Verify layout adaptivity on mobile screens [Browser: Opera]</v>
       </c>
       <c r="C263" t="str">
         <v>Passed</v>
@@ -4868,7 +4868,7 @@
         <v/>
       </c>
       <c r="E263" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.018Z</v>
       </c>
     </row>
     <row r="264">
@@ -4876,7 +4876,7 @@
         <v>TS-WEB-263</v>
       </c>
       <c r="B264" t="str">
-        <v>Verify signup form validation with invalid email [Browser: Mobile Web]</v>
+        <v>Verify layout adaptivity on tablet screens [Browser: Opera]</v>
       </c>
       <c r="C264" t="str">
         <v>Passed</v>
@@ -4885,7 +4885,7 @@
         <v/>
       </c>
       <c r="E264" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.018Z</v>
       </c>
     </row>
     <row r="265">
@@ -4893,7 +4893,7 @@
         <v>TS-WEB-264</v>
       </c>
       <c r="B265" t="str">
-        <v>Verify signup form validation with short password [Browser: Mobile Web]</v>
+        <v>Verify layout adaptivity on 4K desktop screens [Browser: Opera]</v>
       </c>
       <c r="C265" t="str">
         <v>Passed</v>
@@ -4902,7 +4902,7 @@
         <v/>
       </c>
       <c r="E265" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.018Z</v>
       </c>
     </row>
     <row r="266">
@@ -4910,7 +4910,7 @@
         <v>TS-WEB-265</v>
       </c>
       <c r="B266" t="str">
-        <v>Verify signup form verification code (OTP) input format [Browser: Mobile Web]</v>
+        <v>Verify application offline banner displays on network disconnect [Browser: Opera]</v>
       </c>
       <c r="C266" t="str">
         <v>Passed</v>
@@ -4919,7 +4919,7 @@
         <v/>
       </c>
       <c r="E266" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.018Z</v>
       </c>
     </row>
     <row r="267">
@@ -4927,7 +4927,7 @@
         <v>TS-WEB-266</v>
       </c>
       <c r="B267" t="str">
-        <v>Verify login form failure display on bad credentials [Browser: Mobile Web]</v>
+        <v>Verify items with &lt;= 50% freshness have Used/Not Used actions hidden on web [Browser: Opera]</v>
       </c>
       <c r="C267" t="str">
         <v>Passed</v>
@@ -4936,7 +4936,7 @@
         <v/>
       </c>
       <c r="E267" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.018Z</v>
       </c>
     </row>
     <row r="268">
@@ -4944,7 +4944,7 @@
         <v>TS-WEB-267</v>
       </c>
       <c r="B268" t="str">
-        <v>Verify profile update changes reflect immediately on UI [Browser: Mobile Web]</v>
+        <v>Verify items with &lt;= 50% freshness do not generate web recipe recommendations [Browser: Opera]</v>
       </c>
       <c r="C268" t="str">
         <v>Passed</v>
@@ -4953,7 +4953,7 @@
         <v/>
       </c>
       <c r="E268" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.018Z</v>
       </c>
     </row>
     <row r="269">
@@ -4961,7 +4961,7 @@
         <v>TS-WEB-268</v>
       </c>
       <c r="B269" t="str">
-        <v>Verify manual food entry form default category values [Browser: Mobile Web]</v>
+        <v>Verify identical brand logo is displayed across web header layouts [Browser: Opera]</v>
       </c>
       <c r="C269" t="str">
         <v>Passed</v>
@@ -4970,7 +4970,7 @@
         <v/>
       </c>
       <c r="E269" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.018Z</v>
       </c>
     </row>
     <row r="270">
@@ -4978,7 +4978,7 @@
         <v>TS-WEB-269</v>
       </c>
       <c r="B270" t="str">
-        <v>Verify manual food entry fails with empty food name [Browser: Mobile Web]</v>
+        <v>Verify navbar navigation to Dashboard [Browser: Mobile Web]</v>
       </c>
       <c r="C270" t="str">
         <v>Passed</v>
@@ -4987,7 +4987,7 @@
         <v/>
       </c>
       <c r="E270" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.018Z</v>
       </c>
     </row>
     <row r="271">
@@ -4995,7 +4995,7 @@
         <v>TS-WEB-270</v>
       </c>
       <c r="B271" t="str">
-        <v>Verify manual food entry correctly accepts valid dates [Browser: Mobile Web]</v>
+        <v>Verify navbar navigation to Inventory [Browser: Mobile Web]</v>
       </c>
       <c r="C271" t="str">
         <v>Passed</v>
@@ -5004,7 +5004,7 @@
         <v/>
       </c>
       <c r="E271" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.018Z</v>
       </c>
     </row>
     <row r="272">
@@ -5012,7 +5012,7 @@
         <v>TS-WEB-271</v>
       </c>
       <c r="B272" t="str">
-        <v>Verify visual scanner file upload constraints [Browser: Mobile Web]</v>
+        <v>Verify navbar navigation to Scanner [Browser: Mobile Web]</v>
       </c>
       <c r="C272" t="str">
         <v>Passed</v>
@@ -5021,7 +5021,7 @@
         <v/>
       </c>
       <c r="E272" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="273">
@@ -5029,7 +5029,7 @@
         <v>TS-WEB-272</v>
       </c>
       <c r="B273" t="str">
-        <v>Verify visual scanner displays error for non-image files [Browser: Mobile Web]</v>
+        <v>Verify navbar navigation to Analytics [Browser: Mobile Web]</v>
       </c>
       <c r="C273" t="str">
         <v>Passed</v>
@@ -5038,7 +5038,7 @@
         <v/>
       </c>
       <c r="E273" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="274">
@@ -5046,7 +5046,7 @@
         <v>TS-WEB-273</v>
       </c>
       <c r="B274" t="str">
-        <v>Verify OCR scanning auto-populates brand name from image metadata [Browser: Mobile Web]</v>
+        <v>Verify navbar navigation to Household Chores [Browser: Mobile Web]</v>
       </c>
       <c r="C274" t="str">
         <v>Passed</v>
@@ -5055,7 +5055,7 @@
         <v/>
       </c>
       <c r="E274" t="str">
-        <v>2026-08-24T17:52:04.518Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="275">
@@ -5063,7 +5063,7 @@
         <v>TS-WEB-274</v>
       </c>
       <c r="B275" t="str">
-        <v>Verify OCR scanning auto-populates expiry date from label [Browser: Mobile Web]</v>
+        <v>Verify navbar navigation to Neighbor Donations [Browser: Mobile Web]</v>
       </c>
       <c r="C275" t="str">
         <v>Passed</v>
@@ -5072,7 +5072,7 @@
         <v/>
       </c>
       <c r="E275" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="276">
@@ -5080,7 +5080,7 @@
         <v>TS-WEB-275</v>
       </c>
       <c r="B276" t="str">
-        <v>Verify freshness slider adjusts predicted spoilage date [Browser: Mobile Web]</v>
+        <v>Verify navbar navigation to Eco Scorecard [Browser: Mobile Web]</v>
       </c>
       <c r="C276" t="str">
         <v>Passed</v>
@@ -5089,7 +5089,7 @@
         <v/>
       </c>
       <c r="E276" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="277">
@@ -5097,7 +5097,7 @@
         <v>TS-WEB-276</v>
       </c>
       <c r="B277" t="str">
-        <v>Verify CO2 emission indicator increments when food item is marked eaten [Browser: Mobile Web]</v>
+        <v>Verify navbar navigation to Settings [Browser: Mobile Web]</v>
       </c>
       <c r="C277" t="str">
         <v>Passed</v>
@@ -5106,7 +5106,7 @@
         <v/>
       </c>
       <c r="E277" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="278">
@@ -5114,7 +5114,7 @@
         <v>TS-WEB-277</v>
       </c>
       <c r="B278" t="str">
-        <v>Verify streak count updates on daily scanning activity [Browser: Mobile Web]</v>
+        <v>Verify toggle theme between dark and light mode [Browser: Mobile Web]</v>
       </c>
       <c r="C278" t="str">
         <v>Passed</v>
@@ -5123,7 +5123,7 @@
         <v/>
       </c>
       <c r="E278" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="279">
@@ -5131,7 +5131,7 @@
         <v>TS-WEB-278</v>
       </c>
       <c r="B279" t="str">
-        <v>Verify achievement badges render correctly on screen [Browser: Mobile Web]</v>
+        <v>Verify signup form validation with invalid email [Browser: Mobile Web]</v>
       </c>
       <c r="C279" t="str">
         <v>Passed</v>
@@ -5140,7 +5140,7 @@
         <v/>
       </c>
       <c r="E279" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="280">
@@ -5148,7 +5148,7 @@
         <v>TS-WEB-279</v>
       </c>
       <c r="B280" t="str">
-        <v>Verify household join functionality with invalid invite code [Browser: Mobile Web]</v>
+        <v>Verify signup form validation with short password [Browser: Mobile Web]</v>
       </c>
       <c r="C280" t="str">
         <v>Passed</v>
@@ -5157,7 +5157,7 @@
         <v/>
       </c>
       <c r="E280" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="281">
@@ -5165,7 +5165,7 @@
         <v>TS-WEB-280</v>
       </c>
       <c r="B281" t="str">
-        <v>Verify household join succeeds with valid code [Browser: Mobile Web]</v>
+        <v>Verify signup form verification code (OTP) input format [Browser: Mobile Web]</v>
       </c>
       <c r="C281" t="str">
         <v>Passed</v>
@@ -5174,7 +5174,7 @@
         <v/>
       </c>
       <c r="E281" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="282">
@@ -5182,7 +5182,7 @@
         <v>TS-WEB-281</v>
       </c>
       <c r="B282" t="str">
-        <v>Verify household member list loads correctly [Browser: Mobile Web]</v>
+        <v>Verify login form failure display on bad credentials [Browser: Mobile Web]</v>
       </c>
       <c r="C282" t="str">
         <v>Passed</v>
@@ -5191,7 +5191,7 @@
         <v/>
       </c>
       <c r="E282" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="283">
@@ -5199,7 +5199,7 @@
         <v>TS-WEB-282</v>
       </c>
       <c r="B283" t="str">
-        <v>Verify adding household chore updates the task table [Browser: Mobile Web]</v>
+        <v>Verify profile update changes reflect immediately on UI [Browser: Mobile Web]</v>
       </c>
       <c r="C283" t="str">
         <v>Passed</v>
@@ -5208,7 +5208,7 @@
         <v/>
       </c>
       <c r="E283" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="284">
@@ -5216,7 +5216,7 @@
         <v>TS-WEB-283</v>
       </c>
       <c r="B284" t="str">
-        <v>Verify checking household chore changes state to completed [Browser: Mobile Web]</v>
+        <v>Verify manual food entry form default category values [Browser: Mobile Web]</v>
       </c>
       <c r="C284" t="str">
         <v>Passed</v>
@@ -5225,7 +5225,7 @@
         <v/>
       </c>
       <c r="E284" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="285">
@@ -5233,7 +5233,7 @@
         <v>TS-WEB-284</v>
       </c>
       <c r="B285" t="str">
-        <v>Verify neighbor donation list displays available items [Browser: Mobile Web]</v>
+        <v>Verify manual food entry fails with empty food name [Browser: Mobile Web]</v>
       </c>
       <c r="C285" t="str">
         <v>Passed</v>
@@ -5242,7 +5242,7 @@
         <v/>
       </c>
       <c r="E285" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="286">
@@ -5250,7 +5250,7 @@
         <v>TS-WEB-285</v>
       </c>
       <c r="B286" t="str">
-        <v>Verify posting donation item shows up immediately on feed [Browser: Mobile Web]</v>
+        <v>Verify manual food entry correctly accepts valid dates [Browser: Mobile Web]</v>
       </c>
       <c r="C286" t="str">
         <v>Passed</v>
@@ -5259,7 +5259,7 @@
         <v/>
       </c>
       <c r="E286" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="287">
@@ -5267,7 +5267,7 @@
         <v>TS-WEB-286</v>
       </c>
       <c r="B287" t="str">
-        <v>Verify requesting donation item disables button for others [Browser: Mobile Web]</v>
+        <v>Verify visual scanner file upload constraints [Browser: Mobile Web]</v>
       </c>
       <c r="C287" t="str">
         <v>Passed</v>
@@ -5276,7 +5276,7 @@
         <v/>
       </c>
       <c r="E287" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="288">
@@ -5284,7 +5284,7 @@
         <v>TS-WEB-287</v>
       </c>
       <c r="B288" t="str">
-        <v>Verify claiming donation moves item to claimed history [Browser: Mobile Web]</v>
+        <v>Verify visual scanner displays error for non-image files [Browser: Mobile Web]</v>
       </c>
       <c r="C288" t="str">
         <v>Passed</v>
@@ -5293,7 +5293,7 @@
         <v/>
       </c>
       <c r="E288" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="289">
@@ -5301,7 +5301,7 @@
         <v>TS-WEB-288</v>
       </c>
       <c r="B289" t="str">
-        <v>Verify waste report summary matches monthly aggregates [Browser: Mobile Web]</v>
+        <v>Verify OCR scanning auto-populates brand name from image metadata [Browser: Mobile Web]</v>
       </c>
       <c r="C289" t="str">
         <v>Passed</v>
@@ -5310,7 +5310,7 @@
         <v/>
       </c>
       <c r="E289" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="290">
@@ -5318,7 +5318,7 @@
         <v>TS-WEB-289</v>
       </c>
       <c r="B290" t="str">
-        <v>Verify category breakdown chart displays correct percentages [Browser: Mobile Web]</v>
+        <v>Verify OCR scanning auto-populates expiry date from label [Browser: Mobile Web]</v>
       </c>
       <c r="C290" t="str">
         <v>Passed</v>
@@ -5327,7 +5327,7 @@
         <v/>
       </c>
       <c r="E290" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="291">
@@ -5335,7 +5335,7 @@
         <v>TS-WEB-290</v>
       </c>
       <c r="B291" t="str">
-        <v>Verify buy-less smart recommendations update on waste updates [Browser: Mobile Web]</v>
+        <v>Verify freshness slider adjusts predicted spoilage date [Browser: Mobile Web]</v>
       </c>
       <c r="C291" t="str">
         <v>Passed</v>
@@ -5344,7 +5344,7 @@
         <v/>
       </c>
       <c r="E291" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="292">
@@ -5352,7 +5352,7 @@
         <v>TS-WEB-291</v>
       </c>
       <c r="B292" t="str">
-        <v>Verify ambient temperature slider changes shelf-life multipliers [Browser: Mobile Web]</v>
+        <v>Verify CO2 emission indicator increments when food item is marked eaten [Browser: Mobile Web]</v>
       </c>
       <c r="C292" t="str">
         <v>Passed</v>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="E292" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.019Z</v>
       </c>
     </row>
     <row r="293">
@@ -5369,7 +5369,7 @@
         <v>TS-WEB-292</v>
       </c>
       <c r="B293" t="str">
-        <v>Verify custom food item catalog search lists matching records [Browser: Mobile Web]</v>
+        <v>Verify streak count updates on daily scanning activity [Browser: Mobile Web]</v>
       </c>
       <c r="C293" t="str">
         <v>Passed</v>
@@ -5378,7 +5378,7 @@
         <v/>
       </c>
       <c r="E293" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.020Z</v>
       </c>
     </row>
     <row r="294">
@@ -5386,7 +5386,7 @@
         <v>TS-WEB-293</v>
       </c>
       <c r="B294" t="str">
-        <v>Verify notifications panel displays active alerts [Browser: Mobile Web]</v>
+        <v>Verify achievement badges render correctly on screen [Browser: Mobile Web]</v>
       </c>
       <c r="C294" t="str">
         <v>Passed</v>
@@ -5395,7 +5395,7 @@
         <v/>
       </c>
       <c r="E294" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.020Z</v>
       </c>
     </row>
     <row r="295">
@@ -5403,7 +5403,7 @@
         <v>TS-WEB-294</v>
       </c>
       <c r="B295" t="str">
-        <v>Verify critical spoilage alerts display used and waste buttons [Browser: Mobile Web]</v>
+        <v>Verify household join functionality with invalid invite code [Browser: Mobile Web]</v>
       </c>
       <c r="C295" t="str">
         <v>Passed</v>
@@ -5412,7 +5412,7 @@
         <v/>
       </c>
       <c r="E295" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.020Z</v>
       </c>
     </row>
     <row r="296">
@@ -5420,7 +5420,7 @@
         <v>TS-WEB-295</v>
       </c>
       <c r="B296" t="str">
-        <v>Verify clicking used on spoilage alert removes notification [Browser: Mobile Web]</v>
+        <v>Verify household join succeeds with valid code [Browser: Mobile Web]</v>
       </c>
       <c r="C296" t="str">
         <v>Passed</v>
@@ -5429,7 +5429,7 @@
         <v/>
       </c>
       <c r="E296" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.020Z</v>
       </c>
     </row>
     <row r="297">
@@ -5437,7 +5437,7 @@
         <v>TS-WEB-296</v>
       </c>
       <c r="B297" t="str">
-        <v>Verify clicking waste on spoilage alert updates monthly waste [Browser: Mobile Web]</v>
+        <v>Verify household member list loads correctly [Browser: Mobile Web]</v>
       </c>
       <c r="C297" t="str">
         <v>Passed</v>
@@ -5446,7 +5446,7 @@
         <v/>
       </c>
       <c r="E297" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.020Z</v>
       </c>
     </row>
     <row r="298">
@@ -5454,7 +5454,7 @@
         <v>TS-WEB-297</v>
       </c>
       <c r="B298" t="str">
-        <v>Verify email notification preference toggle saves properly [Browser: Mobile Web]</v>
+        <v>Verify adding household chore updates the task table [Browser: Mobile Web]</v>
       </c>
       <c r="C298" t="str">
         <v>Passed</v>
@@ -5463,7 +5463,7 @@
         <v/>
       </c>
       <c r="E298" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.020Z</v>
       </c>
     </row>
     <row r="299">
@@ -5471,7 +5471,7 @@
         <v>TS-WEB-298</v>
       </c>
       <c r="B299" t="str">
-        <v>Verify clear cache utility resets current session state [Browser: Mobile Web]</v>
+        <v>Verify checking household chore changes state to completed [Browser: Mobile Web]</v>
       </c>
       <c r="C299" t="str">
         <v>Passed</v>
@@ -5480,7 +5480,7 @@
         <v/>
       </c>
       <c r="E299" t="str">
-        <v>2026-08-24T17:52:04.519Z</v>
+        <v>2026-08-26T05:28:39.020Z</v>
       </c>
     </row>
     <row r="300">
@@ -5488,7 +5488,7 @@
         <v>TS-WEB-299</v>
       </c>
       <c r="B300" t="str">
-        <v>Verify session persistence on page refresh [Browser: Mobile Web]</v>
+        <v>Verify neighbor donation list displays available items [Browser: Mobile Web]</v>
       </c>
       <c r="C300" t="str">
         <v>Passed</v>
@@ -5497,7 +5497,7 @@
         <v/>
       </c>
       <c r="E300" t="str">
-        <v>2026-08-24T17:52:04.521Z</v>
+        <v>2026-08-26T05:28:39.020Z</v>
       </c>
     </row>
     <row r="301">
@@ -5505,7 +5505,7 @@
         <v>TS-WEB-300</v>
       </c>
       <c r="B301" t="str">
-        <v>Verify layout adaptivity on mobile screens [Browser: Mobile Web]</v>
+        <v>Verify posting donation item shows up immediately on feed [Browser: Mobile Web]</v>
       </c>
       <c r="C301" t="str">
         <v>Passed</v>
@@ -5514,7 +5514,7 @@
         <v/>
       </c>
       <c r="E301" t="str">
-        <v>2026-08-24T17:52:04.521Z</v>
+        <v>2026-08-26T05:28:39.020Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>